<commit_message>
Switch orbital params to SemiMajorAxis and Eccentricity, get load/save to work
</commit_message>
<xml_diff>
--- a/solar-system-generator/Ellipse_Plotter.xlsx
+++ b/solar-system-generator/Ellipse_Plotter.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\source\repos\space-sim\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\source\repos\space-sim\solar-system-generator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9D2605D-4F26-42A2-8502-081C67565918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71D571CB-9035-4A9B-B861-5CF646229F61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-11604" yWindow="648" windowWidth="30984" windowHeight="15864" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="51">
   <si>
     <t>Ellipse calculator</t>
   </si>
@@ -189,6 +189,12 @@
   </si>
   <si>
     <t>Pitch/Orb Inclination</t>
+  </si>
+  <si>
+    <t>Cos(0)</t>
+  </si>
+  <si>
+    <t>Sin(0)</t>
   </si>
 </sst>
 </file>
@@ -392,223 +398,223 @@
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="73"/>
                 <c:pt idx="0">
-                  <c:v>2.4</c:v>
+                  <c:v>1.2000000000000002</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.3772977717989163</c:v>
+                  <c:v>1.1909018964509861</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.3108774751869507</c:v>
+                  <c:v>1.1640842482013765</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2.2054962876570996</c:v>
+                  <c:v>1.1209166818152287</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2.0681731373723151</c:v>
+                  <c:v>1.0634945743553152</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.9071158345178276</c:v>
+                  <c:v>0.99440165299999705</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.7306635447028236</c:v>
+                  <c:v>0.91644952894850895</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.5464550537021053</c:v>
+                  <c:v>0.83243778201311303</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.3609159056305082</c:v>
+                  <c:v>0.74496470040323193</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1.1790518413891289</c:v>
+                  <c:v>0.65630179281363266</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.0044742770028399</c:v>
+                  <c:v>0.56833045227777357</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.83956682871155952</c:v>
+                  <c:v>0.48252969255536332</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.68571428571428583</c:v>
+                  <c:v>0.40000000000000019</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.54353931575946912</c:v>
+                  <c:v>0.32150867592044613</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.41311566495554719</c:v>
+                  <c:v>0.24754472760245377</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.29414438453498853</c:v>
+                  <c:v>0.17837482844585331</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.18609085306989639</c:v>
+                  <c:v>0.11409511062010204</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>8.8286308302482783E-2</c:v>
+                  <c:v>5.4676114325910179E-2</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>5.8807125835613758E-17</c:v>
+                  <c:v>3.6754453647258606E-17</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>-7.9511578622616153E-2</c:v>
+                  <c:v>-5.0109768598056499E-2</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>-0.15097258228534099</c:v>
+                  <c:v>-9.5865474155977376E-2</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>-0.21506805770245765</c:v>
+                  <c:v>-0.13749789067717405</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>-0.27243282855188261</c:v>
+                  <c:v>-0.17524365585003046</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>-0.3236462435502126</c:v>
+                  <c:v>-0.20933628797318143</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>-0.36923076923076908</c:v>
+                  <c:v>-0.23999999999999994</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>-0.40965299566170243</c:v>
+                  <c:v>-0.26744561144535201</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>-0.44532606080535847</c:v>
+                  <c:v>-0.29186799907667815</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>-0.4766128169988848</c:v>
+                  <c:v>-0.31344464995648974</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>-0.50382928908412938</c:v>
+                  <c:v>-0.33233498255227895</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>-0.52724813160591177</c:v>
+                  <c:v>-0.34868018386525329</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>-0.547101900867207</c:v>
+                  <c:v>-0.36260337510235474</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>-0.56358603062362411</c:v>
+                  <c:v>-0.37420996815787883</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>-0.57686144826447339</c:v>
+                  <c:v>-0.38358811291012629</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>-0.58705679902905317</c:v>
+                  <c:v>-0.39080916362535884</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>-0.59427026454600607</c:v>
+                  <c:v>-0.39592811376948212</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>-0.59857097257911507</c:v>
+                  <c:v>-0.3989839640499524</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>-0.6</c:v>
+                  <c:v>-0.40000000000000008</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>-0.59857097257911507</c:v>
+                  <c:v>-0.3989839640499524</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>-0.59427026454600607</c:v>
+                  <c:v>-0.39592811376948212</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>-0.58705679902905317</c:v>
+                  <c:v>-0.39080916362535889</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>-0.5768614482644735</c:v>
+                  <c:v>-0.38358811291012634</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>-0.56358603062362411</c:v>
+                  <c:v>-0.37420996815787888</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>-0.547101900867207</c:v>
+                  <c:v>-0.3626033751023548</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>-0.52724813160591177</c:v>
+                  <c:v>-0.34868018386525323</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>-0.50382928908412938</c:v>
+                  <c:v>-0.332334982552279</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>-0.47661281699888497</c:v>
+                  <c:v>-0.3134446499564898</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>-0.44532606080535853</c:v>
+                  <c:v>-0.29186799907667815</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>-0.40965299566170249</c:v>
+                  <c:v>-0.26744561144535206</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>-0.36923076923076947</c:v>
+                  <c:v>-0.24000000000000021</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>-0.32364624355021249</c:v>
+                  <c:v>-0.20933628797318135</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>-0.2724328285518825</c:v>
+                  <c:v>-0.17524365585003041</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>-0.21506805770245746</c:v>
+                  <c:v>-0.13749789067717394</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>-0.15097258228534102</c:v>
+                  <c:v>-9.5865474155977362E-2</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>-7.9511578622616139E-2</c:v>
+                  <c:v>-5.0109768598056513E-2</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>-1.7642137750684129E-16</c:v>
+                  <c:v>-1.1026336094177581E-16</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>8.8286308302482519E-2</c:v>
+                  <c:v>5.4676114325910012E-2</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>0.1860908530698959</c:v>
+                  <c:v>0.11409511062010173</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>0.29414438453498798</c:v>
+                  <c:v>0.17837482844585298</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>0.41311566495554747</c:v>
+                  <c:v>0.24754472760245388</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>0.54353931575946934</c:v>
+                  <c:v>0.3215086759204463</c:v>
                 </c:pt>
                 <c:pt idx="60">
-                  <c:v>0.68571428571428583</c:v>
+                  <c:v>0.40000000000000019</c:v>
                 </c:pt>
                 <c:pt idx="61">
-                  <c:v>0.83956682871155941</c:v>
+                  <c:v>0.48252969255536327</c:v>
                 </c:pt>
                 <c:pt idx="62">
-                  <c:v>1.0044742770028396</c:v>
+                  <c:v>0.56833045227777346</c:v>
                 </c:pt>
                 <c:pt idx="63">
-                  <c:v>1.179051841389128</c:v>
+                  <c:v>0.65630179281363243</c:v>
                 </c:pt>
                 <c:pt idx="64">
-                  <c:v>1.3609159056305076</c:v>
+                  <c:v>0.74496470040323171</c:v>
                 </c:pt>
                 <c:pt idx="65">
-                  <c:v>1.5464550537021047</c:v>
+                  <c:v>0.83243778201311258</c:v>
                 </c:pt>
                 <c:pt idx="66">
-                  <c:v>1.7306635447028222</c:v>
+                  <c:v>0.91644952894850817</c:v>
                 </c:pt>
                 <c:pt idx="67">
-                  <c:v>1.9071158345178281</c:v>
+                  <c:v>0.99440165299999717</c:v>
                 </c:pt>
                 <c:pt idx="68">
-                  <c:v>2.0681731373723151</c:v>
+                  <c:v>1.0634945743553152</c:v>
                 </c:pt>
                 <c:pt idx="69">
-                  <c:v>2.2054962876570996</c:v>
+                  <c:v>1.1209166818152287</c:v>
                 </c:pt>
                 <c:pt idx="70">
-                  <c:v>2.3108774751869507</c:v>
+                  <c:v>1.1640842482013765</c:v>
                 </c:pt>
                 <c:pt idx="71">
-                  <c:v>2.3772977717989163</c:v>
+                  <c:v>1.1909018964509861</c:v>
                 </c:pt>
                 <c:pt idx="72">
-                  <c:v>2.4</c:v>
+                  <c:v>1.2000000000000002</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -623,220 +629,220 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.20798660485784423</c:v>
+                  <c:v>0.10419041531098511</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.40747004798691572</c:v>
+                  <c:v>0.20525946077563206</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.59096094918755893</c:v>
+                  <c:v>0.30034871967496424</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.75275346131246823</c:v>
+                  <c:v>0.38708036936893925</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.88930271862432397</c:v>
+                  <c:v>0.46369710607588815</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.99919906341084697</c:v>
+                  <c:v>0.5291123822371272</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.0828394861047157</c:v>
+                  <c:v>0.58287921005615284</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.1419440344778533</c:v>
+                  <c:v>0.62509960534844466</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1.1790518413891287</c:v>
+                  <c:v>0.65630179281363255</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.1970858282866059</c:v>
+                  <c:v>0.67730985828272883</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1.199025692951212</c:v>
+                  <c:v>0.68912381861682737</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1.1876919823329444</c:v>
+                  <c:v>0.69282032302755103</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1.1656238242152115</c:v>
+                  <c:v>0.68947758051526153</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1.1350259610883466</c:v>
+                  <c:v>0.68012354939278685</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1.0977617878456545</c:v>
+                  <c:v>0.66570392255130695</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>1.0553736718124536</c:v>
+                  <c:v>0.64706552656705585</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>1.0091171215150916</c:v>
+                  <c:v>0.62495084645691235</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.96</c:v>
+                  <c:v>0.60000000000000009</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.90882150233162262</c:v>
+                  <c:v>0.57275727595505332</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.85620806117559323</c:v>
+                  <c:v>0.54368012070982596</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.80264491843072672</c:v>
+                  <c:v>0.51314911394076446</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.74850304476445018</c:v>
+                  <c:v>0.48147798735063563</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.6940616090903533</c:v>
+                  <c:v>0.44892311827226966</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.63952645202543168</c:v>
+                  <c:v>0.41569219381653066</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>0.58504510921019626</c:v>
+                  <c:v>0.38195191689760538</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0.53071893284061344</c:v>
+                  <c:v>0.34783473646291474</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>0.47661281699888486</c:v>
+                  <c:v>0.3134446499564898</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>0.42276297064680429</c:v>
+                  <c:v>0.27886216128692515</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>0.36918311625744443</c:v>
+                  <c:v>0.24414849316679788</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>0.31586942973983784</c:v>
+                  <c:v>0.2093491562244113</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>0.26280448210897356</c:v>
+                  <c:v>0.17449697390995708</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>0.20996039646396125</c:v>
+                  <c:v>0.1396146553176292</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>0.15730139521103487</c:v>
+                  <c:v>0.10471699978809751</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>0.10478588147221794</c:v>
+                  <c:v>6.9812808878570373E-2</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>5.2368174416359298E-2</c:v>
+                  <c:v>3.490657378300565E-2</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>7.3508907294517201E-17</c:v>
+                  <c:v>4.9005938196344813E-17</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>-5.2368174416359145E-2</c:v>
+                  <c:v>-3.4906573783005553E-2</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>-0.10478588147221807</c:v>
+                  <c:v>-6.9812808878570456E-2</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>-0.15730139521103473</c:v>
+                  <c:v>-0.10471699978809741</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>-0.20996039646396111</c:v>
+                  <c:v>-0.13961465531762912</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>-0.26280448210897334</c:v>
+                  <c:v>-0.174496973909957</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>-0.315869429739838</c:v>
+                  <c:v>-0.20934915622441144</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>-0.36918311625744454</c:v>
+                  <c:v>-0.24414849316679796</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>-0.42276297064680413</c:v>
+                  <c:v>-0.27886216128692509</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>-0.4766128169988848</c:v>
+                  <c:v>-0.31344464995648968</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>-0.53071893284061344</c:v>
+                  <c:v>-0.34783473646291463</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>-0.58504510921019603</c:v>
+                  <c:v>-0.38195191689760527</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>-0.63952645202543124</c:v>
+                  <c:v>-0.41569219381653039</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>-0.6940616090903533</c:v>
+                  <c:v>-0.44892311827226966</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>-0.74850304476445018</c:v>
+                  <c:v>-0.48147798735063574</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>-0.80264491843072672</c:v>
+                  <c:v>-0.51314911394076446</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>-0.85620806117559323</c:v>
+                  <c:v>-0.54368012070982585</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>-0.9088215023316224</c:v>
+                  <c:v>-0.57275727595505332</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>-0.96</c:v>
+                  <c:v>-0.60000000000000009</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>-1.0091171215150914</c:v>
+                  <c:v>-0.62495084645691223</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>-1.0553736718124533</c:v>
+                  <c:v>-0.64706552656705585</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>-1.0977617878456545</c:v>
+                  <c:v>-0.66570392255130684</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>-1.1350259610883469</c:v>
+                  <c:v>-0.68012354939278685</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>-1.1656238242152115</c:v>
+                  <c:v>-0.68947758051526165</c:v>
                 </c:pt>
                 <c:pt idx="60">
-                  <c:v>-1.1876919823329444</c:v>
+                  <c:v>-0.69282032302755103</c:v>
                 </c:pt>
                 <c:pt idx="61">
-                  <c:v>-1.199025692951212</c:v>
+                  <c:v>-0.68912381861682737</c:v>
                 </c:pt>
                 <c:pt idx="62">
-                  <c:v>-1.1970858282866059</c:v>
+                  <c:v>-0.67730985828272894</c:v>
                 </c:pt>
                 <c:pt idx="63">
-                  <c:v>-1.1790518413891287</c:v>
+                  <c:v>-0.65630179281363277</c:v>
                 </c:pt>
                 <c:pt idx="64">
-                  <c:v>-1.1419440344778538</c:v>
+                  <c:v>-0.625099605348445</c:v>
                 </c:pt>
                 <c:pt idx="65">
-                  <c:v>-1.0828394861047161</c:v>
+                  <c:v>-0.58287921005615317</c:v>
                 </c:pt>
                 <c:pt idx="66">
-                  <c:v>-0.99919906341084752</c:v>
+                  <c:v>-0.52911238223712753</c:v>
                 </c:pt>
                 <c:pt idx="67">
-                  <c:v>-0.88930271862432375</c:v>
+                  <c:v>-0.46369710607588793</c:v>
                 </c:pt>
                 <c:pt idx="68">
-                  <c:v>-0.7527534613124679</c:v>
+                  <c:v>-0.38708036936893914</c:v>
                 </c:pt>
                 <c:pt idx="69">
-                  <c:v>-0.5909609491875587</c:v>
+                  <c:v>-0.30034871967496418</c:v>
                 </c:pt>
                 <c:pt idx="70">
-                  <c:v>-0.40747004798691583</c:v>
+                  <c:v>-0.20525946077563212</c:v>
                 </c:pt>
                 <c:pt idx="71">
-                  <c:v>-0.20798660485784459</c:v>
+                  <c:v>-0.10419041531098529</c:v>
                 </c:pt>
                 <c:pt idx="72">
-                  <c:v>-5.8807125835613761E-16</c:v>
+                  <c:v>-2.9403562917806885E-16</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -845,487 +851,6 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000003-194E-48E0-8664-DA386505F5AB}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="5"/>
-          <c:order val="5"/>
-          <c:tx>
-            <c:v>Planet3 Y/Z</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent6"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>Sheet1!$T$9:$T$81</c:f>
-              <c:numCache>
-                <c:formatCode>0.0000</c:formatCode>
-                <c:ptCount val="73"/>
-                <c:pt idx="0">
-                  <c:v>2.4</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>2.3772977717989163</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2.3108774751869507</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>2.2054962876570996</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>2.0681731373723151</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>1.9071158345178276</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>1.7306635447028236</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>1.5464550537021053</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>1.3609159056305082</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>1.1790518413891289</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>1.0044742770028399</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0.83956682871155952</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>0.68571428571428583</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>0.54353931575946912</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>0.41311566495554719</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>0.29414438453498853</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>0.18609085306989639</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>8.8286308302482783E-2</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>5.8807125835613758E-17</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>-7.9511578622616153E-2</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>-0.15097258228534099</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>-0.21506805770245765</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>-0.27243282855188261</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>-0.3236462435502126</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>-0.36923076923076908</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>-0.40965299566170243</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>-0.44532606080535847</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>-0.4766128169988848</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>-0.50382928908412938</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>-0.52724813160591177</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>-0.547101900867207</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>-0.56358603062362411</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>-0.57686144826447339</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>-0.58705679902905317</c:v>
-                </c:pt>
-                <c:pt idx="34">
-                  <c:v>-0.59427026454600607</c:v>
-                </c:pt>
-                <c:pt idx="35">
-                  <c:v>-0.59857097257911507</c:v>
-                </c:pt>
-                <c:pt idx="36">
-                  <c:v>-0.6</c:v>
-                </c:pt>
-                <c:pt idx="37">
-                  <c:v>-0.59857097257911507</c:v>
-                </c:pt>
-                <c:pt idx="38">
-                  <c:v>-0.59427026454600607</c:v>
-                </c:pt>
-                <c:pt idx="39">
-                  <c:v>-0.58705679902905317</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>-0.5768614482644735</c:v>
-                </c:pt>
-                <c:pt idx="41">
-                  <c:v>-0.56358603062362411</c:v>
-                </c:pt>
-                <c:pt idx="42">
-                  <c:v>-0.547101900867207</c:v>
-                </c:pt>
-                <c:pt idx="43">
-                  <c:v>-0.52724813160591177</c:v>
-                </c:pt>
-                <c:pt idx="44">
-                  <c:v>-0.50382928908412938</c:v>
-                </c:pt>
-                <c:pt idx="45">
-                  <c:v>-0.47661281699888497</c:v>
-                </c:pt>
-                <c:pt idx="46">
-                  <c:v>-0.44532606080535853</c:v>
-                </c:pt>
-                <c:pt idx="47">
-                  <c:v>-0.40965299566170249</c:v>
-                </c:pt>
-                <c:pt idx="48">
-                  <c:v>-0.36923076923076947</c:v>
-                </c:pt>
-                <c:pt idx="49">
-                  <c:v>-0.32364624355021249</c:v>
-                </c:pt>
-                <c:pt idx="50">
-                  <c:v>-0.2724328285518825</c:v>
-                </c:pt>
-                <c:pt idx="51">
-                  <c:v>-0.21506805770245746</c:v>
-                </c:pt>
-                <c:pt idx="52">
-                  <c:v>-0.15097258228534102</c:v>
-                </c:pt>
-                <c:pt idx="53">
-                  <c:v>-7.9511578622616139E-2</c:v>
-                </c:pt>
-                <c:pt idx="54">
-                  <c:v>-1.7642137750684129E-16</c:v>
-                </c:pt>
-                <c:pt idx="55">
-                  <c:v>8.8286308302482519E-2</c:v>
-                </c:pt>
-                <c:pt idx="56">
-                  <c:v>0.1860908530698959</c:v>
-                </c:pt>
-                <c:pt idx="57">
-                  <c:v>0.29414438453498798</c:v>
-                </c:pt>
-                <c:pt idx="58">
-                  <c:v>0.41311566495554747</c:v>
-                </c:pt>
-                <c:pt idx="59">
-                  <c:v>0.54353931575946934</c:v>
-                </c:pt>
-                <c:pt idx="60">
-                  <c:v>0.68571428571428583</c:v>
-                </c:pt>
-                <c:pt idx="61">
-                  <c:v>0.83956682871155941</c:v>
-                </c:pt>
-                <c:pt idx="62">
-                  <c:v>1.0044742770028396</c:v>
-                </c:pt>
-                <c:pt idx="63">
-                  <c:v>1.179051841389128</c:v>
-                </c:pt>
-                <c:pt idx="64">
-                  <c:v>1.3609159056305076</c:v>
-                </c:pt>
-                <c:pt idx="65">
-                  <c:v>1.5464550537021047</c:v>
-                </c:pt>
-                <c:pt idx="66">
-                  <c:v>1.7306635447028222</c:v>
-                </c:pt>
-                <c:pt idx="67">
-                  <c:v>1.9071158345178281</c:v>
-                </c:pt>
-                <c:pt idx="68">
-                  <c:v>2.0681731373723151</c:v>
-                </c:pt>
-                <c:pt idx="69">
-                  <c:v>2.2054962876570996</c:v>
-                </c:pt>
-                <c:pt idx="70">
-                  <c:v>2.3108774751869507</c:v>
-                </c:pt>
-                <c:pt idx="71">
-                  <c:v>2.3772977717989163</c:v>
-                </c:pt>
-                <c:pt idx="72">
-                  <c:v>2.4</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>Sheet1!$V$9:$V$81</c:f>
-              <c:numCache>
-                <c:formatCode>0.0000</c:formatCode>
-                <c:ptCount val="73"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="34">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="35">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="36">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="37">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="38">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="39">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="41">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="42">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="43">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="44">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="45">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="46">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="47">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="48">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="49">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="50">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="51">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="52">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="53">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="54">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="55">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="56">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="57">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="58">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="59">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="60">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="61">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="62">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="63">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="64">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="65">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="66">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="67">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="68">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="69">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="70">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="71">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="72">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="1"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-90D6-4034-BE1C-478998149BD9}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1859,7 +1384,7 @@
                 </c:marker>
                 <c:xVal>
                   <c:numRef>
-                    <c:extLst>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                       <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
                           <c15:sqref>Sheet1!$L$9:$L$81</c15:sqref>
@@ -2093,7 +1618,7 @@
                 </c:xVal>
                 <c:yVal>
                   <c:numRef>
-                    <c:extLst>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                       <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
                           <c15:sqref>Sheet1!$M$9:$M$81</c15:sqref>
@@ -2326,7 +1851,7 @@
                   </c:numRef>
                 </c:yVal>
                 <c:smooth val="1"/>
-                <c:extLst>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{00000002-194E-48E0-8664-DA386505F5AB}"/>
                   </c:ext>
@@ -2354,7 +1879,7 @@
                 </c:marker>
                 <c:xVal>
                   <c:numRef>
-                    <c:extLst>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                       <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
                           <c15:sqref>Sheet1!$B$9:$B$81</c15:sqref>
@@ -2588,7 +2113,7 @@
                 </c:xVal>
                 <c:yVal>
                   <c:numRef>
-                    <c:extLst>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                       <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
                           <c15:sqref>Sheet1!$D$9:$D$81</c15:sqref>
@@ -2821,7 +2346,7 @@
                   </c:numRef>
                 </c:yVal>
                 <c:smooth val="1"/>
-                <c:extLst>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{00000000-0156-469D-A974-768DB451DC49}"/>
                   </c:ext>
@@ -2849,7 +2374,7 @@
                 </c:marker>
                 <c:xVal>
                   <c:numRef>
-                    <c:extLst>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                       <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
                           <c15:sqref>Sheet1!$L$9:$L$81</c15:sqref>
@@ -3083,7 +2608,7 @@
                 </c:xVal>
                 <c:yVal>
                   <c:numRef>
-                    <c:extLst>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                       <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
                           <c15:sqref>Sheet1!$N$9:$N$81</c15:sqref>
@@ -3316,9 +2841,504 @@
                   </c:numRef>
                 </c:yVal>
                 <c:smooth val="1"/>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000000-90D6-4034-BE1C-478998149BD9}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="5"/>
+                <c:order val="5"/>
+                <c:tx>
+                  <c:v>Planet3 Y/Z</c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="19050" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent6"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>Sheet1!$T$9:$T$81</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>0.0000</c:formatCode>
+                      <c:ptCount val="73"/>
+                      <c:pt idx="0">
+                        <c:v>1.2000000000000002</c:v>
+                      </c:pt>
+                      <c:pt idx="1">
+                        <c:v>1.1909018964509861</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>1.1640842482013765</c:v>
+                      </c:pt>
+                      <c:pt idx="3">
+                        <c:v>1.1209166818152287</c:v>
+                      </c:pt>
+                      <c:pt idx="4">
+                        <c:v>1.0634945743553152</c:v>
+                      </c:pt>
+                      <c:pt idx="5">
+                        <c:v>0.99440165299999705</c:v>
+                      </c:pt>
+                      <c:pt idx="6">
+                        <c:v>0.91644952894850895</c:v>
+                      </c:pt>
+                      <c:pt idx="7">
+                        <c:v>0.83243778201311303</c:v>
+                      </c:pt>
+                      <c:pt idx="8">
+                        <c:v>0.74496470040323193</c:v>
+                      </c:pt>
+                      <c:pt idx="9">
+                        <c:v>0.65630179281363266</c:v>
+                      </c:pt>
+                      <c:pt idx="10">
+                        <c:v>0.56833045227777357</c:v>
+                      </c:pt>
+                      <c:pt idx="11">
+                        <c:v>0.48252969255536332</c:v>
+                      </c:pt>
+                      <c:pt idx="12">
+                        <c:v>0.40000000000000019</c:v>
+                      </c:pt>
+                      <c:pt idx="13">
+                        <c:v>0.32150867592044613</c:v>
+                      </c:pt>
+                      <c:pt idx="14">
+                        <c:v>0.24754472760245377</c:v>
+                      </c:pt>
+                      <c:pt idx="15">
+                        <c:v>0.17837482844585331</c:v>
+                      </c:pt>
+                      <c:pt idx="16">
+                        <c:v>0.11409511062010204</c:v>
+                      </c:pt>
+                      <c:pt idx="17">
+                        <c:v>5.4676114325910179E-2</c:v>
+                      </c:pt>
+                      <c:pt idx="18">
+                        <c:v>3.6754453647258606E-17</c:v>
+                      </c:pt>
+                      <c:pt idx="19">
+                        <c:v>-5.0109768598056499E-2</c:v>
+                      </c:pt>
+                      <c:pt idx="20">
+                        <c:v>-9.5865474155977376E-2</c:v>
+                      </c:pt>
+                      <c:pt idx="21">
+                        <c:v>-0.13749789067717405</c:v>
+                      </c:pt>
+                      <c:pt idx="22">
+                        <c:v>-0.17524365585003046</c:v>
+                      </c:pt>
+                      <c:pt idx="23">
+                        <c:v>-0.20933628797318143</c:v>
+                      </c:pt>
+                      <c:pt idx="24">
+                        <c:v>-0.23999999999999994</c:v>
+                      </c:pt>
+                      <c:pt idx="25">
+                        <c:v>-0.26744561144535201</c:v>
+                      </c:pt>
+                      <c:pt idx="26">
+                        <c:v>-0.29186799907667815</c:v>
+                      </c:pt>
+                      <c:pt idx="27">
+                        <c:v>-0.31344464995648974</c:v>
+                      </c:pt>
+                      <c:pt idx="28">
+                        <c:v>-0.33233498255227895</c:v>
+                      </c:pt>
+                      <c:pt idx="29">
+                        <c:v>-0.34868018386525329</c:v>
+                      </c:pt>
+                      <c:pt idx="30">
+                        <c:v>-0.36260337510235474</c:v>
+                      </c:pt>
+                      <c:pt idx="31">
+                        <c:v>-0.37420996815787883</c:v>
+                      </c:pt>
+                      <c:pt idx="32">
+                        <c:v>-0.38358811291012629</c:v>
+                      </c:pt>
+                      <c:pt idx="33">
+                        <c:v>-0.39080916362535884</c:v>
+                      </c:pt>
+                      <c:pt idx="34">
+                        <c:v>-0.39592811376948212</c:v>
+                      </c:pt>
+                      <c:pt idx="35">
+                        <c:v>-0.3989839640499524</c:v>
+                      </c:pt>
+                      <c:pt idx="36">
+                        <c:v>-0.40000000000000008</c:v>
+                      </c:pt>
+                      <c:pt idx="37">
+                        <c:v>-0.3989839640499524</c:v>
+                      </c:pt>
+                      <c:pt idx="38">
+                        <c:v>-0.39592811376948212</c:v>
+                      </c:pt>
+                      <c:pt idx="39">
+                        <c:v>-0.39080916362535889</c:v>
+                      </c:pt>
+                      <c:pt idx="40">
+                        <c:v>-0.38358811291012634</c:v>
+                      </c:pt>
+                      <c:pt idx="41">
+                        <c:v>-0.37420996815787888</c:v>
+                      </c:pt>
+                      <c:pt idx="42">
+                        <c:v>-0.3626033751023548</c:v>
+                      </c:pt>
+                      <c:pt idx="43">
+                        <c:v>-0.34868018386525323</c:v>
+                      </c:pt>
+                      <c:pt idx="44">
+                        <c:v>-0.332334982552279</c:v>
+                      </c:pt>
+                      <c:pt idx="45">
+                        <c:v>-0.3134446499564898</c:v>
+                      </c:pt>
+                      <c:pt idx="46">
+                        <c:v>-0.29186799907667815</c:v>
+                      </c:pt>
+                      <c:pt idx="47">
+                        <c:v>-0.26744561144535206</c:v>
+                      </c:pt>
+                      <c:pt idx="48">
+                        <c:v>-0.24000000000000021</c:v>
+                      </c:pt>
+                      <c:pt idx="49">
+                        <c:v>-0.20933628797318135</c:v>
+                      </c:pt>
+                      <c:pt idx="50">
+                        <c:v>-0.17524365585003041</c:v>
+                      </c:pt>
+                      <c:pt idx="51">
+                        <c:v>-0.13749789067717394</c:v>
+                      </c:pt>
+                      <c:pt idx="52">
+                        <c:v>-9.5865474155977362E-2</c:v>
+                      </c:pt>
+                      <c:pt idx="53">
+                        <c:v>-5.0109768598056513E-2</c:v>
+                      </c:pt>
+                      <c:pt idx="54">
+                        <c:v>-1.1026336094177581E-16</c:v>
+                      </c:pt>
+                      <c:pt idx="55">
+                        <c:v>5.4676114325910012E-2</c:v>
+                      </c:pt>
+                      <c:pt idx="56">
+                        <c:v>0.11409511062010173</c:v>
+                      </c:pt>
+                      <c:pt idx="57">
+                        <c:v>0.17837482844585298</c:v>
+                      </c:pt>
+                      <c:pt idx="58">
+                        <c:v>0.24754472760245388</c:v>
+                      </c:pt>
+                      <c:pt idx="59">
+                        <c:v>0.3215086759204463</c:v>
+                      </c:pt>
+                      <c:pt idx="60">
+                        <c:v>0.40000000000000019</c:v>
+                      </c:pt>
+                      <c:pt idx="61">
+                        <c:v>0.48252969255536327</c:v>
+                      </c:pt>
+                      <c:pt idx="62">
+                        <c:v>0.56833045227777346</c:v>
+                      </c:pt>
+                      <c:pt idx="63">
+                        <c:v>0.65630179281363243</c:v>
+                      </c:pt>
+                      <c:pt idx="64">
+                        <c:v>0.74496470040323171</c:v>
+                      </c:pt>
+                      <c:pt idx="65">
+                        <c:v>0.83243778201311258</c:v>
+                      </c:pt>
+                      <c:pt idx="66">
+                        <c:v>0.91644952894850817</c:v>
+                      </c:pt>
+                      <c:pt idx="67">
+                        <c:v>0.99440165299999717</c:v>
+                      </c:pt>
+                      <c:pt idx="68">
+                        <c:v>1.0634945743553152</c:v>
+                      </c:pt>
+                      <c:pt idx="69">
+                        <c:v>1.1209166818152287</c:v>
+                      </c:pt>
+                      <c:pt idx="70">
+                        <c:v>1.1640842482013765</c:v>
+                      </c:pt>
+                      <c:pt idx="71">
+                        <c:v>1.1909018964509861</c:v>
+                      </c:pt>
+                      <c:pt idx="72">
+                        <c:v>1.2000000000000002</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>Sheet1!$V$9:$V$81</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>0.0000</c:formatCode>
+                      <c:ptCount val="73"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="1">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="3">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="4">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="5">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="6">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="7">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="8">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="9">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="10">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="11">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="12">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="13">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="14">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="15">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="16">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="17">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="18">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="19">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="20">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="21">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="22">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="23">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="24">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="25">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="26">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="27">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="28">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="29">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="30">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="31">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="32">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="33">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="34">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="35">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="36">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="37">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="38">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="39">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="40">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="41">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="42">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="43">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="44">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="45">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="46">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="47">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="48">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="49">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="50">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="51">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="52">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="53">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="54">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="55">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="56">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="57">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="58">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="59">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="60">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="61">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="62">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="63">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="64">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="65">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="66">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="67">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="68">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="69">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="70">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="71">
+                        <c:v>0</c:v>
+                      </c:pt>
+                      <c:pt idx="72">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="1"/>
                 <c:extLst>
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000000-90D6-4034-BE1C-478998149BD9}"/>
+                    <c16:uniqueId val="{00000001-90D6-4034-BE1C-478998149BD9}"/>
                   </c:ext>
                 </c:extLst>
               </c15:ser>
@@ -4457,6 +4477,13 @@
       <c r="U2" t="s">
         <v>46</v>
       </c>
+      <c r="AB2" t="s">
+        <v>49</v>
+      </c>
+      <c r="AC2">
+        <f>COS(0)</f>
+        <v>1</v>
+      </c>
       <c r="AF2" t="s">
         <v>19</v>
       </c>
@@ -4506,7 +4533,7 @@
         <v>4</v>
       </c>
       <c r="T3" s="7">
-        <v>1.5</v>
+        <v>0.8</v>
       </c>
       <c r="U3" t="s">
         <v>7</v>
@@ -4516,7 +4543,14 @@
       </c>
       <c r="W3">
         <f>T$3*(1-T$6^2)</f>
-        <v>0.96</v>
+        <v>0.60000000000000009</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>50</v>
+      </c>
+      <c r="AC3">
+        <f>SIN(0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:35" x14ac:dyDescent="0.3">
@@ -4567,7 +4601,7 @@
       </c>
       <c r="T4">
         <f>SQRT((1-T6^2)*T3^2)</f>
-        <v>1.2</v>
+        <v>0.69282032302755103</v>
       </c>
       <c r="U4" t="s">
         <v>7</v>
@@ -4577,7 +4611,7 @@
       </c>
       <c r="W4" s="1">
         <f>-0.0000000000667*2E+30/(2*T$3*150000000000)</f>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333337</v>
       </c>
       <c r="X4" t="s">
         <v>17</v>
@@ -4651,7 +4685,7 @@
       </c>
       <c r="T5">
         <f>SQRT(T3^2-T4^2)</f>
-        <v>0.9</v>
+        <v>0.39999999999999997</v>
       </c>
       <c r="U5" t="s">
         <v>7</v>
@@ -4733,7 +4767,7 @@
         <v>6</v>
       </c>
       <c r="T6" s="7">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="V6" t="s">
         <v>48</v>
@@ -4991,7 +5025,7 @@
       </c>
       <c r="T9" s="4">
         <f>W9*COS(RADIANS(S9))*(COS($Y$5)*COS($Y$6))+W9*SIN(RADIANS(S9))*(COS($Y$5)*SIN($Y$6)*SIN($Y$7)-SIN($Y$5)*COS($Y$7))</f>
-        <v>2.4</v>
+        <v>1.2000000000000002</v>
       </c>
       <c r="U9" s="4">
         <f>W9*COS(RADIANS(S9))*(SIN(Y$5)*COS(Y$6))+W9*SIN(RADIANS(S9))*(SIN(Y$5)*SIN(Y$6)*SIN(Y$7)+COS(Y$5)*COS(Y$7))</f>
@@ -5003,23 +5037,23 @@
       </c>
       <c r="W9" s="5">
         <f>W$3/(1-T$6*COS(RADIANS(S9)))</f>
-        <v>2.4</v>
+        <v>1.2000000000000002</v>
       </c>
       <c r="X9" s="2">
         <f>SQRT(0.0000000000667*2E+30/(W9*150000000000))</f>
-        <v>19249.819623974548</v>
+        <v>27223.355985460556</v>
       </c>
       <c r="Y9" s="1">
         <f>W$4-Z9</f>
-        <v>-481722222.22222221</v>
+        <v>-926388888.88888884</v>
       </c>
       <c r="Z9" s="1">
         <f>X9^2/2</f>
-        <v>185277777.77777782</v>
+        <v>370555555.55555552</v>
       </c>
       <c r="AA9" s="1">
         <f>SUM(Y9:Z9)</f>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="10" spans="1:35" x14ac:dyDescent="0.3">
@@ -5098,11 +5132,11 @@
       </c>
       <c r="T10" s="4">
         <f t="shared" ref="T10:T73" si="17">W10*COS(RADIANS(S10))*(COS($Y$5)*COS($Y$6))+W10*SIN(RADIANS(S10))*(COS($Y$5)*SIN($Y$6)*SIN($Y$7)-SIN($Y$5)*COS($Y$7))</f>
-        <v>2.3772977717989163</v>
+        <v>1.1909018964509861</v>
       </c>
       <c r="U10" s="4">
         <f t="shared" ref="U10:U73" si="18">W10*COS(RADIANS(S10))*(SIN(Y$5)*COS(Y$6))+W10*SIN(RADIANS(S10))*(SIN(Y$5)*SIN(Y$6)*SIN(Y$7)+COS(Y$5)*COS(Y$7))</f>
-        <v>0.20798660485784423</v>
+        <v>0.10419041531098511</v>
       </c>
       <c r="V10" s="4">
         <f t="shared" ref="V10:V73" si="19">W10*COS(RADIANS(S10))*(-SIN(Y$6))+W10*SIN(RADIANS(S10))*(COS(Y$6)*SIN(Y$7))</f>
@@ -5110,23 +5144,23 @@
       </c>
       <c r="W10" s="5">
         <f t="shared" ref="W10:W12" si="20">W$3/(1-T$6*COS(RADIANS(S10)))</f>
-        <v>2.3863786630793498</v>
+        <v>1.1954509482254931</v>
       </c>
       <c r="X10" s="2">
         <f t="shared" ref="X10:X73" si="21">SQRT(0.0000000000667*2E+30/(W10*150000000000))</f>
-        <v>19304.679981796133</v>
+        <v>27275.103347860128</v>
       </c>
       <c r="Y10" s="1">
         <f t="shared" ref="Y10:Y34" si="22">W$4-Z10</f>
-        <v>-482779779.04422462</v>
+        <v>-927798964.65155876</v>
       </c>
       <c r="Z10" s="1">
         <f t="shared" ref="Z10:Z34" si="23">X10^2/2</f>
-        <v>186335334.59978017</v>
+        <v>371965631.31822538</v>
       </c>
       <c r="AA10" s="1">
         <f t="shared" ref="AA10:AA34" si="24">SUM(Y10:Z10)</f>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="11" spans="1:35" x14ac:dyDescent="0.3">
@@ -5205,11 +5239,11 @@
       </c>
       <c r="T11" s="4">
         <f t="shared" si="17"/>
-        <v>2.3108774751869507</v>
+        <v>1.1640842482013765</v>
       </c>
       <c r="U11" s="4">
         <f t="shared" si="18"/>
-        <v>0.40747004798691572</v>
+        <v>0.20525946077563206</v>
       </c>
       <c r="V11" s="4">
         <f t="shared" si="19"/>
@@ -5217,23 +5251,23 @@
       </c>
       <c r="W11" s="5">
         <f t="shared" si="20"/>
-        <v>2.3465264851121703</v>
+        <v>1.1820421241006884</v>
       </c>
       <c r="X11" s="2">
         <f t="shared" si="21"/>
-        <v>19467.920095367233</v>
+        <v>27429.368460766789</v>
       </c>
       <c r="Y11" s="1">
         <f t="shared" si="22"/>
-        <v>-485944400.86424613</v>
+        <v>-932018460.41158724</v>
       </c>
       <c r="Z11" s="1">
         <f t="shared" si="23"/>
-        <v>189499956.41980168</v>
+        <v>376185127.07825392</v>
       </c>
       <c r="AA11" s="1">
         <f t="shared" si="24"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="12" spans="1:35" x14ac:dyDescent="0.3">
@@ -5312,11 +5346,11 @@
       </c>
       <c r="T12" s="4">
         <f t="shared" si="17"/>
-        <v>2.2054962876570996</v>
+        <v>1.1209166818152287</v>
       </c>
       <c r="U12" s="4">
         <f t="shared" si="18"/>
-        <v>0.59096094918755893</v>
+        <v>0.30034871967496424</v>
       </c>
       <c r="V12" s="4">
         <f t="shared" si="19"/>
@@ -5324,23 +5358,23 @@
       </c>
       <c r="W12" s="5">
         <f t="shared" si="20"/>
-        <v>2.2832977725942598</v>
+        <v>1.1604583409076143</v>
       </c>
       <c r="X12" s="2">
         <f t="shared" si="21"/>
-        <v>19735.630648902043</v>
+        <v>27683.277621159901</v>
       </c>
       <c r="Y12" s="1">
         <f t="shared" si="22"/>
-        <v>-491192002.99938524</v>
+        <v>-939015263.25843966</v>
       </c>
       <c r="Z12" s="1">
         <f t="shared" si="23"/>
-        <v>194747558.55494082</v>
+        <v>383181929.92510629</v>
       </c>
       <c r="AA12" s="1">
         <f t="shared" si="24"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="13" spans="1:35" x14ac:dyDescent="0.3">
@@ -5419,11 +5453,11 @@
       </c>
       <c r="T13" s="4">
         <f t="shared" si="17"/>
-        <v>2.0681731373723151</v>
+        <v>1.0634945743553152</v>
       </c>
       <c r="U13" s="4">
         <f t="shared" si="18"/>
-        <v>0.75275346131246823</v>
+        <v>0.38708036936893925</v>
       </c>
       <c r="V13" s="4">
         <f t="shared" si="19"/>
@@ -5431,23 +5465,23 @@
       </c>
       <c r="W13" s="5">
         <f t="shared" ref="W13:W76" si="25">W$3/(1-T$6*COS(RADIANS(S13)))</f>
-        <v>2.2009038824233889</v>
+        <v>1.1317472871776577</v>
       </c>
       <c r="X13" s="2">
         <f t="shared" si="21"/>
-        <v>20101.651851743965</v>
+        <v>28032.223956166334</v>
       </c>
       <c r="Y13" s="1">
         <f t="shared" si="22"/>
-        <v>-498482648.02880526</v>
+        <v>-948736123.29766619</v>
       </c>
       <c r="Z13" s="1">
         <f t="shared" si="23"/>
-        <v>202038203.58436081</v>
+        <v>392902789.96433282</v>
       </c>
       <c r="AA13" s="1">
         <f t="shared" si="24"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.3">
@@ -5526,11 +5560,11 @@
       </c>
       <c r="T14" s="4">
         <f t="shared" si="17"/>
-        <v>1.9071158345178276</v>
+        <v>0.99440165299999705</v>
       </c>
       <c r="U14" s="4">
         <f t="shared" si="18"/>
-        <v>0.88930271862432397</v>
+        <v>0.46369710607588815</v>
       </c>
       <c r="V14" s="4">
         <f t="shared" si="19"/>
@@ -5538,23 +5572,23 @@
       </c>
       <c r="W14" s="5">
         <f t="shared" si="25"/>
-        <v>2.1042695007106964</v>
+        <v>1.0972008264999986</v>
       </c>
       <c r="X14" s="2">
         <f t="shared" si="21"/>
-        <v>20558.0351832161</v>
+        <v>28470.115053558147</v>
       </c>
       <c r="Y14" s="1">
         <f t="shared" si="22"/>
-        <v>-507760849.74161994</v>
+        <v>-961107058.91475248</v>
       </c>
       <c r="Z14" s="1">
         <f t="shared" si="23"/>
-        <v>211316405.2971755</v>
+        <v>405273725.58141911</v>
       </c>
       <c r="AA14" s="1">
         <f t="shared" si="24"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.3">
@@ -5633,11 +5667,11 @@
       </c>
       <c r="T15" s="4">
         <f t="shared" si="17"/>
-        <v>1.7306635447028236</v>
+        <v>0.91644952894850895</v>
       </c>
       <c r="U15" s="4">
         <f t="shared" si="18"/>
-        <v>0.99919906341084697</v>
+        <v>0.5291123822371272</v>
       </c>
       <c r="V15" s="4">
         <f t="shared" si="19"/>
@@ -5645,23 +5679,23 @@
       </c>
       <c r="W15" s="5">
         <f t="shared" si="25"/>
-        <v>1.9983981268216942</v>
+        <v>1.0582247644742546</v>
       </c>
       <c r="X15" s="2">
         <f t="shared" si="21"/>
-        <v>21095.570671400154</v>
+        <v>28989.67355754611</v>
       </c>
       <c r="Y15" s="1">
         <f t="shared" si="22"/>
-        <v>-518955995.42046356</v>
+        <v>-976033919.81987739</v>
       </c>
       <c r="Z15" s="1">
         <f t="shared" si="23"/>
-        <v>222511550.97601917</v>
+        <v>420200586.48654407</v>
       </c>
       <c r="AA15" s="1">
         <f t="shared" si="24"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="16" spans="1:35" x14ac:dyDescent="0.3">
@@ -5740,11 +5774,11 @@
       </c>
       <c r="T16" s="4">
         <f t="shared" si="17"/>
-        <v>1.5464550537021053</v>
+        <v>0.83243778201311303</v>
       </c>
       <c r="U16" s="4">
         <f t="shared" si="18"/>
-        <v>1.0828394861047157</v>
+        <v>0.58287921005615284</v>
       </c>
       <c r="V16" s="4">
         <f t="shared" si="19"/>
@@ -5752,23 +5786,23 @@
       </c>
       <c r="W16" s="5">
         <f t="shared" si="25"/>
-        <v>1.8878730322212631</v>
+        <v>1.0162188910065566</v>
       </c>
       <c r="X16" s="2">
         <f t="shared" si="21"/>
-        <v>21704.305508468231</v>
+        <v>29582.757486587845</v>
       </c>
       <c r="Y16" s="1">
         <f t="shared" si="22"/>
-        <v>-531982883.24690664</v>
+        <v>-993403103.58846796</v>
       </c>
       <c r="Z16" s="1">
         <f t="shared" si="23"/>
-        <v>235538438.80246219</v>
+        <v>437569770.25513458</v>
       </c>
       <c r="AA16" s="1">
         <f t="shared" si="24"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.3">
@@ -5847,11 +5881,11 @@
       </c>
       <c r="T17" s="4">
         <f t="shared" si="17"/>
-        <v>1.3609159056305082</v>
+        <v>0.74496470040323193</v>
       </c>
       <c r="U17" s="4">
         <f t="shared" si="18"/>
-        <v>1.1419440344778533</v>
+        <v>0.62509960534844466</v>
       </c>
       <c r="V17" s="4">
         <f t="shared" si="19"/>
@@ -5859,23 +5893,23 @@
       </c>
       <c r="W17" s="5">
         <f t="shared" si="25"/>
-        <v>1.776549543378305</v>
+        <v>0.972482350201616</v>
       </c>
       <c r="X17" s="2">
         <f t="shared" si="21"/>
-        <v>22373.999476816618</v>
+        <v>30240.670856014818</v>
       </c>
       <c r="Y17" s="1">
         <f t="shared" si="22"/>
-        <v>-546742370.73873961</v>
+        <v>-1013082420.2442453</v>
       </c>
       <c r="Z17" s="1">
         <f t="shared" si="23"/>
-        <v>250297926.29429516</v>
+        <v>457249086.91091198</v>
       </c>
       <c r="AA17" s="1">
         <f t="shared" si="24"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.3">
@@ -5954,11 +5988,11 @@
       </c>
       <c r="T18" s="4">
         <f t="shared" si="17"/>
-        <v>1.1790518413891289</v>
+        <v>0.65630179281363266</v>
       </c>
       <c r="U18" s="4">
         <f t="shared" si="18"/>
-        <v>1.1790518413891287</v>
+        <v>0.65630179281363255</v>
       </c>
       <c r="V18" s="4">
         <f t="shared" si="19"/>
@@ -5966,23 +6000,23 @@
       </c>
       <c r="W18" s="5">
         <f t="shared" si="25"/>
-        <v>1.6674311048334773</v>
+        <v>0.92815089640681636</v>
       </c>
       <c r="X18" s="2">
         <f t="shared" si="21"/>
-        <v>23094.487863543676</v>
+        <v>30954.442814285296</v>
       </c>
       <c r="Y18" s="1">
         <f t="shared" si="22"/>
-        <v>-563122129.28412747</v>
+        <v>-1034922098.3047626</v>
       </c>
       <c r="Z18" s="1">
         <f t="shared" si="23"/>
-        <v>266677684.83968309</v>
+        <v>479088764.97142929</v>
       </c>
       <c r="AA18" s="1">
         <f t="shared" si="24"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.3">
@@ -6061,11 +6095,11 @@
       </c>
       <c r="T19" s="4">
         <f t="shared" si="17"/>
-        <v>1.0044742770028399</v>
+        <v>0.56833045227777357</v>
       </c>
       <c r="U19" s="4">
         <f t="shared" si="18"/>
-        <v>1.1970858282866059</v>
+        <v>0.67730985828272883</v>
       </c>
       <c r="V19" s="4">
         <f t="shared" si="19"/>
@@ -6073,23 +6107,23 @@
       </c>
       <c r="W19" s="5">
         <f t="shared" si="25"/>
-        <v>1.5626845662017037</v>
+        <v>0.88416522613888682</v>
       </c>
       <c r="X19" s="2">
         <f t="shared" si="21"/>
-        <v>23855.944944006184</v>
+        <v>31715.062393111821</v>
       </c>
       <c r="Y19" s="1">
         <f t="shared" si="22"/>
-        <v>-580997499.03017151</v>
+        <v>-1058755924.6328212</v>
       </c>
       <c r="Z19" s="1">
         <f t="shared" si="23"/>
-        <v>284553054.5857271</v>
+        <v>502922591.29948783</v>
       </c>
       <c r="AA19" s="1">
         <f t="shared" si="24"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.3">
@@ -6168,11 +6202,11 @@
       </c>
       <c r="T20" s="4">
         <f t="shared" si="17"/>
-        <v>0.83956682871155952</v>
+        <v>0.48252969255536332</v>
       </c>
       <c r="U20" s="4">
         <f t="shared" si="18"/>
-        <v>1.199025692951212</v>
+        <v>0.68912381861682737</v>
       </c>
       <c r="V20" s="4">
         <f t="shared" si="19"/>
@@ -6180,23 +6214,23 @@
       </c>
       <c r="W20" s="5">
         <f t="shared" si="25"/>
-        <v>1.4637400972269357</v>
+        <v>0.84126484627768172</v>
       </c>
       <c r="X20" s="2">
         <f t="shared" si="21"/>
-        <v>24649.05650020772</v>
+        <v>32513.664084057749</v>
       </c>
       <c r="Y20" s="1">
         <f t="shared" si="22"/>
-        <v>-600232437.61966062</v>
+        <v>-1084402509.4188068</v>
       </c>
       <c r="Z20" s="1">
         <f t="shared" si="23"/>
-        <v>303787993.17521626</v>
+        <v>528569176.08547342</v>
       </c>
       <c r="AA20" s="1">
         <f t="shared" si="24"/>
-        <v>-296444444.44444436</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.3">
@@ -6275,11 +6309,11 @@
       </c>
       <c r="T21" s="4">
         <f t="shared" si="17"/>
-        <v>0.68571428571428583</v>
+        <v>0.40000000000000019</v>
       </c>
       <c r="U21" s="4">
         <f t="shared" si="18"/>
-        <v>1.1876919823329444</v>
+        <v>0.69282032302755103</v>
       </c>
       <c r="V21" s="4">
         <f t="shared" si="19"/>
@@ -6287,23 +6321,23 @@
       </c>
       <c r="W21" s="5">
         <f t="shared" si="25"/>
-        <v>1.3714285714285714</v>
+        <v>0.80000000000000016</v>
       </c>
       <c r="X21" s="2">
         <f t="shared" si="21"/>
-        <v>25465.11775394377</v>
+        <v>33341.665625260328</v>
       </c>
       <c r="Y21" s="1">
         <f t="shared" si="22"/>
-        <v>-620680555.55555558</v>
+        <v>-1111666666.6666665</v>
       </c>
       <c r="Z21" s="1">
         <f t="shared" si="23"/>
-        <v>324236111.1111111</v>
+        <v>555833333.33333313</v>
       </c>
       <c r="AA21" s="1">
         <f t="shared" si="24"/>
-        <v>-296444444.44444448</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.3">
@@ -6382,11 +6416,11 @@
       </c>
       <c r="T22" s="4">
         <f t="shared" si="17"/>
-        <v>0.54353931575946912</v>
+        <v>0.32150867592044613</v>
       </c>
       <c r="U22" s="4">
         <f t="shared" si="18"/>
-        <v>1.1656238242152115</v>
+        <v>0.68947758051526153</v>
       </c>
       <c r="V22" s="4">
         <f t="shared" si="19"/>
@@ -6394,23 +6428,23 @@
       </c>
       <c r="W22" s="5">
         <f t="shared" si="25"/>
-        <v>1.2861235894556815</v>
+        <v>0.76075433796022318</v>
       </c>
       <c r="X22" s="2">
         <f t="shared" si="21"/>
-        <v>26296.075215476867</v>
+        <v>34190.86329251904</v>
       </c>
       <c r="Y22" s="1">
         <f t="shared" si="22"/>
-        <v>-642186230.31345272</v>
+        <v>-1140340899.6771963</v>
       </c>
       <c r="Z22" s="1">
         <f t="shared" si="23"/>
-        <v>345741785.86900836</v>
+        <v>584507566.34386289</v>
       </c>
       <c r="AA22" s="1">
         <f t="shared" si="24"/>
-        <v>-296444444.44444436</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.3">
@@ -6489,11 +6523,11 @@
       </c>
       <c r="T23" s="4">
         <f t="shared" si="17"/>
-        <v>0.41311566495554719</v>
+        <v>0.24754472760245377</v>
       </c>
       <c r="U23" s="4">
         <f t="shared" si="18"/>
-        <v>1.1350259610883466</v>
+        <v>0.68012354939278685</v>
       </c>
       <c r="V23" s="4">
         <f t="shared" si="19"/>
@@ -6501,23 +6535,23 @@
       </c>
       <c r="W23" s="5">
         <f t="shared" si="25"/>
-        <v>1.2078693989733282</v>
+        <v>0.723772363801227</v>
       </c>
       <c r="X23" s="2">
         <f t="shared" si="21"/>
-        <v>27134.529525256894</v>
+        <v>35053.491891390135</v>
       </c>
       <c r="Y23" s="1">
         <f t="shared" si="22"/>
-        <v>-664585790.72296345</v>
+        <v>-1170206980.2232103</v>
       </c>
       <c r="Z23" s="1">
         <f t="shared" si="23"/>
-        <v>368141346.27851903</v>
+        <v>614373646.88987696</v>
       </c>
       <c r="AA23" s="1">
         <f t="shared" si="24"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.3">
@@ -6596,11 +6630,11 @@
       </c>
       <c r="T24" s="4">
         <f t="shared" si="17"/>
-        <v>0.29414438453498853</v>
+        <v>0.17837482844585331</v>
       </c>
       <c r="U24" s="4">
         <f t="shared" si="18"/>
-        <v>1.0977617878456545</v>
+        <v>0.66570392255130695</v>
       </c>
       <c r="V24" s="4">
         <f t="shared" si="19"/>
@@ -6608,23 +6642,23 @@
       </c>
       <c r="W24" s="5">
         <f t="shared" si="25"/>
-        <v>1.1364866307209931</v>
+        <v>0.68918741422292673</v>
       </c>
       <c r="X24" s="2">
         <f t="shared" si="21"/>
-        <v>27973.713309451865</v>
+        <v>35922.257057840565</v>
       </c>
       <c r="Y24" s="1">
         <f t="shared" si="22"/>
-        <v>-687708762.6041466</v>
+        <v>-1201037609.3981214</v>
       </c>
       <c r="Z24" s="1">
         <f t="shared" si="23"/>
-        <v>391264318.15970218</v>
+        <v>645204276.0647881</v>
       </c>
       <c r="AA24" s="1">
         <f t="shared" si="24"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.3">
@@ -6703,11 +6737,11 @@
       </c>
       <c r="T25" s="4">
         <f t="shared" si="17"/>
-        <v>0.18609085306989639</v>
+        <v>0.11409511062010204</v>
       </c>
       <c r="U25" s="4">
         <f t="shared" si="18"/>
-        <v>1.0553736718124536</v>
+        <v>0.64706552656705585</v>
       </c>
       <c r="V25" s="4">
         <f t="shared" si="19"/>
@@ -6715,23 +6749,23 @@
       </c>
       <c r="W25" s="5">
         <f t="shared" si="25"/>
-        <v>1.0716545118419378</v>
+        <v>0.6570475553100511</v>
       </c>
       <c r="X25" s="2">
         <f t="shared" si="21"/>
-        <v>28807.45465099303</v>
+        <v>36790.346944940102</v>
       </c>
       <c r="Y25" s="1">
         <f t="shared" si="22"/>
-        <v>-711379166.17895436</v>
+        <v>-1232598147.4978652</v>
       </c>
       <c r="Z25" s="1">
         <f t="shared" si="23"/>
-        <v>414934721.73450994</v>
+        <v>676764814.16453171</v>
       </c>
       <c r="AA25" s="1">
         <f t="shared" si="24"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333349</v>
       </c>
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.3">
@@ -6810,11 +6844,11 @@
       </c>
       <c r="T26" s="4">
         <f t="shared" si="17"/>
-        <v>8.8286308302482783E-2</v>
+        <v>5.4676114325910179E-2</v>
       </c>
       <c r="U26" s="4">
         <f t="shared" si="18"/>
-        <v>1.0091171215150916</v>
+        <v>0.62495084645691235</v>
       </c>
       <c r="V26" s="4">
         <f t="shared" si="19"/>
@@ -6822,23 +6856,23 @@
       </c>
       <c r="W26" s="5">
         <f t="shared" si="25"/>
-        <v>1.0129717849814897</v>
+        <v>0.62733805716295521</v>
       </c>
       <c r="X26" s="2">
         <f t="shared" si="21"/>
-        <v>29630.133679724018</v>
+        <v>37651.429360315007</v>
       </c>
       <c r="Y26" s="1">
         <f t="shared" si="22"/>
-        <v>-735416855.38360214</v>
+        <v>-1264648399.7707288</v>
       </c>
       <c r="Z26" s="1">
         <f t="shared" si="23"/>
-        <v>438972410.93915778</v>
+        <v>708815066.43739545</v>
       </c>
       <c r="AA26" s="1">
         <f t="shared" si="24"/>
-        <v>-296444444.44444436</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="27" spans="1:27" x14ac:dyDescent="0.3">
@@ -6917,11 +6951,11 @@
       </c>
       <c r="T27" s="4">
         <f t="shared" si="17"/>
-        <v>5.8807125835613758E-17</v>
+        <v>3.6754453647258606E-17</v>
       </c>
       <c r="U27" s="4">
         <f t="shared" si="18"/>
-        <v>0.96</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="V27" s="4">
         <f t="shared" si="19"/>
@@ -6929,23 +6963,23 @@
       </c>
       <c r="W27" s="5">
         <f t="shared" si="25"/>
-        <v>0.96</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="X27" s="2">
         <f t="shared" si="21"/>
-        <v>30436.637279582788</v>
+        <v>38499.63924794909</v>
       </c>
       <c r="Y27" s="1">
         <f t="shared" si="22"/>
-        <v>-759638888.88888884</v>
+        <v>-1296944444.4444442</v>
       </c>
       <c r="Z27" s="1">
         <f t="shared" si="23"/>
-        <v>463194444.44444436</v>
+        <v>741111111.11111093</v>
       </c>
       <c r="AA27" s="1">
         <f t="shared" si="24"/>
-        <v>-296444444.44444448</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="28" spans="1:27" x14ac:dyDescent="0.3">
@@ -7024,11 +7058,11 @@
       </c>
       <c r="T28" s="4">
         <f t="shared" si="17"/>
-        <v>-7.9511578622616153E-2</v>
+        <v>-5.0109768598056499E-2</v>
       </c>
       <c r="U28" s="4">
         <f t="shared" si="18"/>
-        <v>0.90882150233162262</v>
+        <v>0.57275727595505332</v>
       </c>
       <c r="V28" s="4">
         <f t="shared" si="19"/>
@@ -7036,23 +7070,23 @@
       </c>
       <c r="W28" s="5">
         <f t="shared" si="25"/>
-        <v>0.91229305282643036</v>
+        <v>0.57494511570097184</v>
       </c>
       <c r="X28" s="2">
         <f t="shared" si="21"/>
-        <v>31222.315031071321</v>
+        <v>39329.560276840792</v>
       </c>
       <c r="Y28" s="1">
         <f t="shared" si="22"/>
-        <v>-783860922.39417553</v>
+        <v>-1329240489.1181598</v>
       </c>
       <c r="Z28" s="1">
         <f t="shared" si="23"/>
-        <v>487416477.94973105</v>
+        <v>773407155.78482652</v>
       </c>
       <c r="AA28" s="1">
         <f t="shared" si="24"/>
-        <v>-296444444.44444448</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="29" spans="1:27" x14ac:dyDescent="0.3">
@@ -7131,11 +7165,11 @@
       </c>
       <c r="T29" s="4">
         <f t="shared" si="17"/>
-        <v>-0.15097258228534099</v>
+        <v>-9.5865474155977376E-2</v>
       </c>
       <c r="U29" s="4">
         <f t="shared" si="18"/>
-        <v>0.85620806117559323</v>
+        <v>0.54368012070982596</v>
       </c>
       <c r="V29" s="4">
         <f t="shared" si="19"/>
@@ -7143,23 +7177,23 @@
       </c>
       <c r="W29" s="5">
         <f t="shared" si="25"/>
-        <v>0.86941645062879536</v>
+        <v>0.55206726292201147</v>
       </c>
       <c r="X29" s="2">
         <f t="shared" si="21"/>
-        <v>31982.938175045107</v>
+        <v>40136.203309672681</v>
       </c>
       <c r="Y29" s="1">
         <f t="shared" si="22"/>
-        <v>-807898611.59882331</v>
+        <v>-1361290741.3910236</v>
       </c>
       <c r="Z29" s="1">
         <f t="shared" si="23"/>
-        <v>511454167.15437883</v>
+        <v>805457408.05769014</v>
       </c>
       <c r="AA29" s="1">
         <f t="shared" si="24"/>
-        <v>-296444444.44444448</v>
+        <v>-555833333.33333349</v>
       </c>
     </row>
     <row r="30" spans="1:27" x14ac:dyDescent="0.3">
@@ -7238,11 +7272,11 @@
       </c>
       <c r="T30" s="4">
         <f t="shared" si="17"/>
-        <v>-0.21506805770245765</v>
+        <v>-0.13749789067717405</v>
       </c>
       <c r="U30" s="4">
         <f t="shared" si="18"/>
-        <v>0.80264491843072672</v>
+        <v>0.51314911394076446</v>
       </c>
       <c r="V30" s="4">
         <f t="shared" si="19"/>
@@ -7250,23 +7284,23 @@
       </c>
       <c r="W30" s="5">
         <f t="shared" si="25"/>
-        <v>0.83095916537852543</v>
+        <v>0.53125105466141309</v>
       </c>
       <c r="X30" s="2">
         <f t="shared" si="21"/>
-        <v>32714.662484249679</v>
+        <v>40914.983713975351</v>
       </c>
       <c r="Y30" s="1">
         <f t="shared" si="22"/>
-        <v>-831569015.17363107</v>
+        <v>-1392851279.4907675</v>
       </c>
       <c r="Z30" s="1">
         <f t="shared" si="23"/>
-        <v>535124570.72918665</v>
+        <v>837017946.15743411</v>
       </c>
       <c r="AA30" s="1">
         <f t="shared" si="24"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="31" spans="1:27" x14ac:dyDescent="0.3">
@@ -7345,11 +7379,11 @@
       </c>
       <c r="T31" s="4">
         <f t="shared" si="17"/>
-        <v>-0.27243282855188261</v>
+        <v>-0.17524365585003046</v>
       </c>
       <c r="U31" s="4">
         <f t="shared" si="18"/>
-        <v>0.74850304476445018</v>
+        <v>0.48147798735063563</v>
       </c>
       <c r="V31" s="4">
         <f t="shared" si="19"/>
@@ -7357,23 +7391,23 @@
       </c>
       <c r="W31" s="5">
         <f t="shared" si="25"/>
-        <v>0.79654030286887045</v>
+        <v>0.51237817207498482</v>
       </c>
       <c r="X31" s="2">
         <f t="shared" si="21"/>
-        <v>33413.995349564822</v>
+        <v>41661.698845158608</v>
       </c>
       <c r="Y31" s="1">
         <f t="shared" si="22"/>
-        <v>-854691987.05481422</v>
+        <v>-1423681908.6656785</v>
       </c>
       <c r="Z31" s="1">
         <f t="shared" si="23"/>
-        <v>558247542.6103698</v>
+        <v>867848575.33234501</v>
       </c>
       <c r="AA31" s="1">
         <f t="shared" si="24"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333349</v>
       </c>
     </row>
     <row r="32" spans="1:27" x14ac:dyDescent="0.3">
@@ -7452,11 +7486,11 @@
       </c>
       <c r="T32" s="4">
         <f t="shared" si="17"/>
-        <v>-0.3236462435502126</v>
+        <v>-0.20933628797318143</v>
       </c>
       <c r="U32" s="4">
         <f t="shared" si="18"/>
-        <v>0.6940616090903533</v>
+        <v>0.44892311827226966</v>
       </c>
       <c r="V32" s="4">
         <f t="shared" si="19"/>
@@ -7464,23 +7498,23 @@
       </c>
       <c r="W32" s="5">
         <f t="shared" si="25"/>
-        <v>0.76581225386987239</v>
+        <v>0.4953318560134094</v>
       </c>
       <c r="X32" s="2">
         <f t="shared" si="21"/>
-        <v>34077.767034237455</v>
+        <v>42372.506555037762</v>
       </c>
       <c r="Y32" s="1">
         <f t="shared" si="22"/>
-        <v>-877091547.46432495</v>
+        <v>-1453547989.2116923</v>
       </c>
       <c r="Z32" s="1">
         <f t="shared" si="23"/>
-        <v>580647103.01988053</v>
+        <v>897714655.87835908</v>
       </c>
       <c r="AA32" s="1">
         <f t="shared" si="24"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="33" spans="1:27" x14ac:dyDescent="0.3">
@@ -7559,11 +7593,11 @@
       </c>
       <c r="T33" s="4">
         <f t="shared" si="17"/>
-        <v>-0.36923076923076908</v>
+        <v>-0.23999999999999994</v>
       </c>
       <c r="U33" s="4">
         <f t="shared" si="18"/>
-        <v>0.63952645202543168</v>
+        <v>0.41569219381653066</v>
       </c>
       <c r="V33" s="4">
         <f t="shared" si="19"/>
@@ -7571,23 +7605,23 @@
       </c>
       <c r="W33" s="5">
         <f t="shared" si="25"/>
-        <v>0.7384615384615385</v>
+        <v>0.48000000000000009</v>
       </c>
       <c r="X33" s="2">
         <f t="shared" si="21"/>
-        <v>34703.105848836582</v>
+        <v>43043.90523381652</v>
       </c>
       <c r="Y33" s="1">
         <f t="shared" si="22"/>
-        <v>-898597222.22222233</v>
+        <v>-1482222222.2222219</v>
       </c>
       <c r="Z33" s="1">
         <f t="shared" si="23"/>
-        <v>602152777.77777791</v>
+        <v>926388888.8888886</v>
       </c>
       <c r="AA33" s="1">
         <f t="shared" si="24"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="34" spans="1:27" x14ac:dyDescent="0.3">
@@ -7666,11 +7700,11 @@
       </c>
       <c r="T34" s="4">
         <f t="shared" si="17"/>
-        <v>-0.40965299566170243</v>
+        <v>-0.26744561144535201</v>
       </c>
       <c r="U34" s="4">
         <f t="shared" si="18"/>
-        <v>0.58504510921019626</v>
+        <v>0.38195191689760538</v>
       </c>
       <c r="V34" s="4">
         <f t="shared" si="19"/>
@@ -7678,23 +7712,23 @@
       </c>
       <c r="W34" s="5">
         <f t="shared" si="25"/>
-        <v>0.71420820260297857</v>
+        <v>0.46627719427732411</v>
       </c>
       <c r="X34" s="2">
         <f t="shared" si="21"/>
-        <v>35287.416899333184</v>
+        <v>43672.715650317616</v>
       </c>
       <c r="Y34" s="1">
         <f t="shared" si="22"/>
-        <v>-919045340.15811706</v>
+        <v>-1509486379.4700818</v>
       </c>
       <c r="Z34" s="1">
         <f t="shared" si="23"/>
-        <v>622600895.71367264</v>
+        <v>953653046.13674855</v>
       </c>
       <c r="AA34" s="1">
         <f t="shared" si="24"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="35" spans="1:27" x14ac:dyDescent="0.3">
@@ -7773,11 +7807,11 @@
       </c>
       <c r="T35" s="4">
         <f t="shared" si="17"/>
-        <v>-0.44532606080535847</v>
+        <v>-0.29186799907667815</v>
       </c>
       <c r="U35" s="4">
         <f t="shared" si="18"/>
-        <v>0.53071893284061344</v>
+        <v>0.34783473646291474</v>
       </c>
       <c r="V35" s="4">
         <f t="shared" si="19"/>
@@ -7785,23 +7819,23 @@
       </c>
       <c r="W35" s="5">
         <f t="shared" si="25"/>
-        <v>0.69280436351678487</v>
+        <v>0.45406600046166101</v>
       </c>
       <c r="X35" s="2">
         <f t="shared" si="21"/>
-        <v>35828.36402358226</v>
+        <v>44256.064690000043</v>
       </c>
       <c r="Y35" s="1">
         <f t="shared" ref="Y35:Y81" si="32">W$4-Z35</f>
-        <v>-938280278.74760628</v>
+        <v>-1535132964.2560678</v>
       </c>
       <c r="Z35" s="1">
         <f t="shared" ref="Z35:Z81" si="33">X35^2/2</f>
-        <v>641835834.30316186</v>
+        <v>979299630.92273426</v>
       </c>
       <c r="AA35" s="1">
         <f t="shared" ref="AA35:AA81" si="34">SUM(Y35:Z35)</f>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333349</v>
       </c>
     </row>
     <row r="36" spans="1:27" x14ac:dyDescent="0.3">
@@ -7880,11 +7914,11 @@
       </c>
       <c r="T36" s="4">
         <f t="shared" si="17"/>
-        <v>-0.4766128169988848</v>
+        <v>-0.31344464995648974</v>
       </c>
       <c r="U36" s="4">
         <f t="shared" si="18"/>
-        <v>0.47661281699888486</v>
+        <v>0.3134446499564898</v>
       </c>
       <c r="V36" s="4">
         <f t="shared" si="19"/>
@@ -7892,23 +7926,23 @@
       </c>
       <c r="W36" s="5">
         <f t="shared" si="25"/>
-        <v>0.67403230980066897</v>
+        <v>0.44327767502175519</v>
       </c>
       <c r="X36" s="2">
         <f t="shared" si="21"/>
-        <v>36323.854532502628</v>
+        <v>44791.370982607637</v>
       </c>
       <c r="Y36" s="1">
         <f t="shared" si="32"/>
-        <v>-956155648.49365032</v>
+        <v>-1558966790.584126</v>
       </c>
       <c r="Z36" s="1">
         <f t="shared" si="33"/>
-        <v>659711204.0492059</v>
+        <v>1003133457.2507927</v>
       </c>
       <c r="AA36" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="37" spans="1:27" x14ac:dyDescent="0.3">
@@ -7987,11 +8021,11 @@
       </c>
       <c r="T37" s="4">
         <f t="shared" si="17"/>
-        <v>-0.50382928908412938</v>
+        <v>-0.33233498255227895</v>
       </c>
       <c r="U37" s="4">
         <f t="shared" si="18"/>
-        <v>0.42276297064680429</v>
+        <v>0.27886216128692515</v>
       </c>
       <c r="V37" s="4">
         <f t="shared" si="19"/>
@@ -7999,23 +8033,23 @@
       </c>
       <c r="W37" s="5">
         <f t="shared" si="25"/>
-        <v>0.65770242654952238</v>
+        <v>0.43383250872386064</v>
       </c>
       <c r="X37" s="2">
         <f t="shared" si="21"/>
-        <v>36772.026394926725</v>
+        <v>45276.332345085328</v>
       </c>
       <c r="Y37" s="1">
         <f t="shared" si="32"/>
-        <v>-972535407.0390383</v>
+        <v>-1580806468.6446433</v>
       </c>
       <c r="Z37" s="1">
         <f t="shared" si="33"/>
-        <v>676090962.59459388</v>
+        <v>1024973135.3113099</v>
       </c>
       <c r="AA37" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="38" spans="1:27" x14ac:dyDescent="0.3">
@@ -8094,11 +8128,11 @@
       </c>
       <c r="T38" s="4">
         <f t="shared" si="17"/>
-        <v>-0.52724813160591177</v>
+        <v>-0.34868018386525329</v>
       </c>
       <c r="U38" s="4">
         <f t="shared" si="18"/>
-        <v>0.36918311625744443</v>
+        <v>0.24414849316679788</v>
       </c>
       <c r="V38" s="4">
         <f t="shared" si="19"/>
@@ -8106,23 +8140,23 @@
       </c>
       <c r="W38" s="5">
         <f t="shared" si="25"/>
-        <v>0.64365112103645294</v>
+        <v>0.42565990806737342</v>
       </c>
       <c r="X38" s="2">
         <f t="shared" si="21"/>
-        <v>37171.237538893613</v>
+        <v>45708.914928426981</v>
       </c>
       <c r="Y38" s="1">
         <f t="shared" si="32"/>
-        <v>-987294894.53087127</v>
+        <v>-1600485785.3004208</v>
       </c>
       <c r="Z38" s="1">
         <f t="shared" si="33"/>
-        <v>690850450.08642685</v>
+        <v>1044652451.9670874</v>
       </c>
       <c r="AA38" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="39" spans="1:27" x14ac:dyDescent="0.3">
@@ -8201,11 +8235,11 @@
       </c>
       <c r="T39" s="4">
         <f t="shared" si="17"/>
-        <v>-0.547101900867207</v>
+        <v>-0.36260337510235474</v>
       </c>
       <c r="U39" s="4">
         <f t="shared" si="18"/>
-        <v>0.31586942973983784</v>
+        <v>0.2093491562244113</v>
       </c>
       <c r="V39" s="4">
         <f t="shared" si="19"/>
@@ -8213,23 +8247,23 @@
       </c>
       <c r="W39" s="5">
         <f t="shared" si="25"/>
-        <v>0.63173885947967579</v>
+        <v>0.41869831244882266</v>
       </c>
       <c r="X39" s="2">
         <f t="shared" si="21"/>
-        <v>37520.056980576926</v>
+        <v>46087.343940298364</v>
       </c>
       <c r="Y39" s="1">
         <f t="shared" si="32"/>
-        <v>-1000321782.3573141</v>
+        <v>-1617854969.0690117</v>
       </c>
       <c r="Z39" s="1">
         <f t="shared" si="33"/>
-        <v>703877337.91286969</v>
+        <v>1062021635.7356782</v>
       </c>
       <c r="AA39" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333349</v>
       </c>
     </row>
     <row r="40" spans="1:27" x14ac:dyDescent="0.3">
@@ -8308,11 +8342,11 @@
       </c>
       <c r="T40" s="4">
         <f t="shared" si="17"/>
-        <v>-0.56358603062362411</v>
+        <v>-0.37420996815787883</v>
       </c>
       <c r="U40" s="4">
         <f t="shared" si="18"/>
-        <v>0.26280448210897356</v>
+        <v>0.17449697390995708</v>
       </c>
       <c r="V40" s="4">
         <f t="shared" si="19"/>
@@ -8320,23 +8354,23 @@
       </c>
       <c r="W40" s="5">
         <f t="shared" si="25"/>
-        <v>0.62184838162582556</v>
+        <v>0.41289501592106065</v>
       </c>
       <c r="X40" s="2">
         <f t="shared" si="21"/>
-        <v>37817.257531230724</v>
+        <v>46410.095812027866</v>
       </c>
       <c r="Y40" s="1">
         <f t="shared" si="32"/>
-        <v>-1011516928.0361578</v>
+        <v>-1632781829.9741368</v>
       </c>
       <c r="Z40" s="1">
         <f t="shared" si="33"/>
-        <v>715072483.59171343</v>
+        <v>1076948496.6408033</v>
       </c>
       <c r="AA40" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333349</v>
       </c>
     </row>
     <row r="41" spans="1:27" x14ac:dyDescent="0.3">
@@ -8415,11 +8449,11 @@
       </c>
       <c r="T41" s="4">
         <f t="shared" si="17"/>
-        <v>-0.57686144826447339</v>
+        <v>-0.38358811291012629</v>
       </c>
       <c r="U41" s="4">
         <f t="shared" si="18"/>
-        <v>0.20996039646396125</v>
+        <v>0.1396146553176292</v>
       </c>
       <c r="V41" s="4">
         <f t="shared" si="19"/>
@@ -8427,23 +8461,23 @@
       </c>
       <c r="W41" s="5">
         <f t="shared" si="25"/>
-        <v>0.61388313104131598</v>
+        <v>0.40820594354493689</v>
       </c>
       <c r="X41" s="2">
         <f t="shared" si="21"/>
-        <v>38061.809870381308</v>
+        <v>46675.891684206508</v>
       </c>
       <c r="Y41" s="1">
         <f t="shared" si="32"/>
-        <v>-1020795129.7489724</v>
+        <v>-1645152765.5912223</v>
       </c>
       <c r="Z41" s="1">
         <f t="shared" si="33"/>
-        <v>724350685.304528</v>
+        <v>1089319432.257889</v>
       </c>
       <c r="AA41" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="42" spans="1:27" x14ac:dyDescent="0.3">
@@ -8522,11 +8556,11 @@
       </c>
       <c r="T42" s="4">
         <f t="shared" si="17"/>
-        <v>-0.58705679902905317</v>
+        <v>-0.39080916362535884</v>
       </c>
       <c r="U42" s="4">
         <f t="shared" si="18"/>
-        <v>0.15730139521103487</v>
+        <v>0.10471699978809751</v>
       </c>
       <c r="V42" s="4">
         <f t="shared" si="19"/>
@@ -8534,23 +8568,23 @@
       </c>
       <c r="W42" s="5">
         <f t="shared" si="25"/>
-        <v>0.60776592058256795</v>
+        <v>0.4045954181873207</v>
       </c>
       <c r="X42" s="2">
         <f t="shared" si="21"/>
-        <v>38252.877808968784</v>
+        <v>46883.692096444698</v>
       </c>
       <c r="Y42" s="1">
         <f t="shared" si="32"/>
-        <v>-1028085774.7783927</v>
+        <v>-1654873625.6304488</v>
       </c>
       <c r="Z42" s="1">
         <f t="shared" si="33"/>
-        <v>731641330.33394825</v>
+        <v>1099040292.2971156</v>
       </c>
       <c r="AA42" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="43" spans="1:27" x14ac:dyDescent="0.3">
@@ -8629,11 +8663,11 @@
       </c>
       <c r="T43" s="4">
         <f t="shared" si="17"/>
-        <v>-0.59427026454600607</v>
+        <v>-0.39592811376948212</v>
       </c>
       <c r="U43" s="4">
         <f t="shared" si="18"/>
-        <v>0.10478588147221794</v>
+        <v>6.9812808878570373E-2</v>
       </c>
       <c r="V43" s="4">
         <f t="shared" si="19"/>
@@ -8641,23 +8675,23 @@
       </c>
       <c r="W43" s="5">
         <f t="shared" si="25"/>
-        <v>0.6034378412723963</v>
+        <v>0.40203594311525903</v>
       </c>
       <c r="X43" s="2">
         <f t="shared" si="21"/>
-        <v>38389.814598903373</v>
+        <v>47032.692781595397</v>
       </c>
       <c r="Y43" s="1">
         <f t="shared" si="32"/>
-        <v>-1033333376.9135317</v>
+        <v>-1661870428.4773011</v>
       </c>
       <c r="Z43" s="1">
         <f t="shared" si="33"/>
-        <v>736888932.46908724</v>
+        <v>1106037095.1439679</v>
       </c>
       <c r="AA43" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="44" spans="1:27" x14ac:dyDescent="0.3">
@@ -8736,11 +8770,11 @@
       </c>
       <c r="T44" s="4">
         <f t="shared" si="17"/>
-        <v>-0.59857097257911507</v>
+        <v>-0.3989839640499524</v>
       </c>
       <c r="U44" s="4">
         <f t="shared" si="18"/>
-        <v>5.2368174416359298E-2</v>
+        <v>3.490657378300565E-2</v>
       </c>
       <c r="V44" s="4">
         <f t="shared" si="19"/>
@@ -8748,23 +8782,23 @@
       </c>
       <c r="W44" s="5">
         <f t="shared" si="25"/>
-        <v>0.60085741645253077</v>
+        <v>0.40050801797502394</v>
       </c>
       <c r="X44" s="2">
         <f t="shared" si="21"/>
-        <v>38472.160175615529</v>
+        <v>47122.321481522886</v>
       </c>
       <c r="Y44" s="1">
         <f t="shared" si="32"/>
-        <v>-1036497998.7335532</v>
+        <v>-1666089924.23733</v>
       </c>
       <c r="Z44" s="1">
         <f t="shared" si="33"/>
-        <v>740053554.28910875</v>
+        <v>1110256590.9039967</v>
       </c>
       <c r="AA44" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="45" spans="1:27" x14ac:dyDescent="0.3">
@@ -8843,11 +8877,11 @@
       </c>
       <c r="T45" s="4">
         <f t="shared" si="17"/>
-        <v>-0.6</v>
+        <v>-0.40000000000000008</v>
       </c>
       <c r="U45" s="4">
         <f t="shared" si="18"/>
-        <v>7.3508907294517201E-17</v>
+        <v>4.9005938196344813E-17</v>
       </c>
       <c r="V45" s="4">
         <f t="shared" si="19"/>
@@ -8855,23 +8889,23 @@
       </c>
       <c r="W45" s="5">
         <f t="shared" si="25"/>
-        <v>0.6</v>
+        <v>0.40000000000000008</v>
       </c>
       <c r="X45" s="2">
         <f t="shared" si="21"/>
-        <v>38499.639247949097</v>
+        <v>47152.235719351978</v>
       </c>
       <c r="Y45" s="1">
         <f t="shared" si="32"/>
-        <v>-1037555555.5555557</v>
+        <v>-1667499999.9999995</v>
       </c>
       <c r="Z45" s="1">
         <f t="shared" si="33"/>
-        <v>741111111.11111128</v>
+        <v>1111666666.6666663</v>
       </c>
       <c r="AA45" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="46" spans="1:27" x14ac:dyDescent="0.3">
@@ -8950,11 +8984,11 @@
       </c>
       <c r="T46" s="4">
         <f t="shared" si="17"/>
-        <v>-0.59857097257911507</v>
+        <v>-0.3989839640499524</v>
       </c>
       <c r="U46" s="4">
         <f t="shared" si="18"/>
-        <v>-5.2368174416359145E-2</v>
+        <v>-3.4906573783005553E-2</v>
       </c>
       <c r="V46" s="4">
         <f t="shared" si="19"/>
@@ -8962,23 +8996,23 @@
       </c>
       <c r="W46" s="5">
         <f t="shared" si="25"/>
-        <v>0.60085741645253077</v>
+        <v>0.40050801797502394</v>
       </c>
       <c r="X46" s="2">
         <f t="shared" si="21"/>
-        <v>38472.160175615529</v>
+        <v>47122.321481522886</v>
       </c>
       <c r="Y46" s="1">
         <f t="shared" si="32"/>
-        <v>-1036497998.7335532</v>
+        <v>-1666089924.23733</v>
       </c>
       <c r="Z46" s="1">
         <f t="shared" si="33"/>
-        <v>740053554.28910875</v>
+        <v>1110256590.9039967</v>
       </c>
       <c r="AA46" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="47" spans="1:27" x14ac:dyDescent="0.3">
@@ -9057,11 +9091,11 @@
       </c>
       <c r="T47" s="4">
         <f t="shared" si="17"/>
-        <v>-0.59427026454600607</v>
+        <v>-0.39592811376948212</v>
       </c>
       <c r="U47" s="4">
         <f t="shared" si="18"/>
-        <v>-0.10478588147221807</v>
+        <v>-6.9812808878570456E-2</v>
       </c>
       <c r="V47" s="4">
         <f t="shared" si="19"/>
@@ -9069,23 +9103,23 @@
       </c>
       <c r="W47" s="5">
         <f t="shared" si="25"/>
-        <v>0.6034378412723963</v>
+        <v>0.40203594311525903</v>
       </c>
       <c r="X47" s="2">
         <f t="shared" si="21"/>
-        <v>38389.814598903373</v>
+        <v>47032.692781595397</v>
       </c>
       <c r="Y47" s="1">
         <f t="shared" si="32"/>
-        <v>-1033333376.9135317</v>
+        <v>-1661870428.4773011</v>
       </c>
       <c r="Z47" s="1">
         <f t="shared" si="33"/>
-        <v>736888932.46908724</v>
+        <v>1106037095.1439679</v>
       </c>
       <c r="AA47" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="48" spans="1:27" x14ac:dyDescent="0.3">
@@ -9164,11 +9198,11 @@
       </c>
       <c r="T48" s="4">
         <f t="shared" si="17"/>
-        <v>-0.58705679902905317</v>
+        <v>-0.39080916362535889</v>
       </c>
       <c r="U48" s="4">
         <f t="shared" si="18"/>
-        <v>-0.15730139521103473</v>
+        <v>-0.10471699978809741</v>
       </c>
       <c r="V48" s="4">
         <f t="shared" si="19"/>
@@ -9176,23 +9210,23 @@
       </c>
       <c r="W48" s="5">
         <f t="shared" si="25"/>
-        <v>0.60776592058256795</v>
+        <v>0.4045954181873207</v>
       </c>
       <c r="X48" s="2">
         <f t="shared" si="21"/>
-        <v>38252.877808968784</v>
+        <v>46883.692096444698</v>
       </c>
       <c r="Y48" s="1">
         <f t="shared" si="32"/>
-        <v>-1028085774.7783927</v>
+        <v>-1654873625.6304488</v>
       </c>
       <c r="Z48" s="1">
         <f t="shared" si="33"/>
-        <v>731641330.33394825</v>
+        <v>1099040292.2971156</v>
       </c>
       <c r="AA48" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="49" spans="1:27" x14ac:dyDescent="0.3">
@@ -9271,11 +9305,11 @@
       </c>
       <c r="T49" s="4">
         <f t="shared" si="17"/>
-        <v>-0.5768614482644735</v>
+        <v>-0.38358811291012634</v>
       </c>
       <c r="U49" s="4">
         <f t="shared" si="18"/>
-        <v>-0.20996039646396111</v>
+        <v>-0.13961465531762912</v>
       </c>
       <c r="V49" s="4">
         <f t="shared" si="19"/>
@@ -9283,23 +9317,23 @@
       </c>
       <c r="W49" s="5">
         <f t="shared" si="25"/>
-        <v>0.61388313104131598</v>
+        <v>0.40820594354493689</v>
       </c>
       <c r="X49" s="2">
         <f t="shared" si="21"/>
-        <v>38061.809870381308</v>
+        <v>46675.891684206508</v>
       </c>
       <c r="Y49" s="1">
         <f t="shared" si="32"/>
-        <v>-1020795129.7489724</v>
+        <v>-1645152765.5912223</v>
       </c>
       <c r="Z49" s="1">
         <f t="shared" si="33"/>
-        <v>724350685.304528</v>
+        <v>1089319432.257889</v>
       </c>
       <c r="AA49" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="50" spans="1:27" x14ac:dyDescent="0.3">
@@ -9378,11 +9412,11 @@
       </c>
       <c r="T50" s="4">
         <f t="shared" si="17"/>
-        <v>-0.56358603062362411</v>
+        <v>-0.37420996815787888</v>
       </c>
       <c r="U50" s="4">
         <f t="shared" si="18"/>
-        <v>-0.26280448210897334</v>
+        <v>-0.174496973909957</v>
       </c>
       <c r="V50" s="4">
         <f t="shared" si="19"/>
@@ -9390,23 +9424,23 @@
       </c>
       <c r="W50" s="5">
         <f t="shared" si="25"/>
-        <v>0.62184838162582545</v>
+        <v>0.41289501592106065</v>
       </c>
       <c r="X50" s="2">
         <f t="shared" si="21"/>
-        <v>37817.257531230724</v>
+        <v>46410.095812027866</v>
       </c>
       <c r="Y50" s="1">
         <f t="shared" si="32"/>
-        <v>-1011516928.0361578</v>
+        <v>-1632781829.9741368</v>
       </c>
       <c r="Z50" s="1">
         <f t="shared" si="33"/>
-        <v>715072483.59171343</v>
+        <v>1076948496.6408033</v>
       </c>
       <c r="AA50" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333349</v>
       </c>
     </row>
     <row r="51" spans="1:27" x14ac:dyDescent="0.3">
@@ -9485,11 +9519,11 @@
       </c>
       <c r="T51" s="4">
         <f t="shared" si="17"/>
-        <v>-0.547101900867207</v>
+        <v>-0.3626033751023548</v>
       </c>
       <c r="U51" s="4">
         <f t="shared" si="18"/>
-        <v>-0.315869429739838</v>
+        <v>-0.20934915622441144</v>
       </c>
       <c r="V51" s="4">
         <f t="shared" si="19"/>
@@ -9497,23 +9531,23 @@
       </c>
       <c r="W51" s="5">
         <f t="shared" si="25"/>
-        <v>0.6317388594796759</v>
+        <v>0.41869831244882277</v>
       </c>
       <c r="X51" s="2">
         <f t="shared" si="21"/>
-        <v>37520.056980576926</v>
+        <v>46087.343940298357</v>
       </c>
       <c r="Y51" s="1">
         <f t="shared" si="32"/>
-        <v>-1000321782.3573141</v>
+        <v>-1617854969.0690112</v>
       </c>
       <c r="Z51" s="1">
         <f t="shared" si="33"/>
-        <v>703877337.91286969</v>
+        <v>1062021635.7356778</v>
       </c>
       <c r="AA51" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="52" spans="1:27" x14ac:dyDescent="0.3">
@@ -9592,11 +9626,11 @@
       </c>
       <c r="T52" s="4">
         <f t="shared" si="17"/>
-        <v>-0.52724813160591177</v>
+        <v>-0.34868018386525323</v>
       </c>
       <c r="U52" s="4">
         <f t="shared" si="18"/>
-        <v>-0.36918311625744454</v>
+        <v>-0.24414849316679796</v>
       </c>
       <c r="V52" s="4">
         <f t="shared" si="19"/>
@@ -9604,23 +9638,23 @@
       </c>
       <c r="W52" s="5">
         <f t="shared" si="25"/>
-        <v>0.64365112103645294</v>
+        <v>0.42565990806737342</v>
       </c>
       <c r="X52" s="2">
         <f t="shared" si="21"/>
-        <v>37171.237538893613</v>
+        <v>45708.914928426981</v>
       </c>
       <c r="Y52" s="1">
         <f t="shared" si="32"/>
-        <v>-987294894.53087127</v>
+        <v>-1600485785.3004208</v>
       </c>
       <c r="Z52" s="1">
         <f t="shared" si="33"/>
-        <v>690850450.08642685</v>
+        <v>1044652451.9670874</v>
       </c>
       <c r="AA52" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="53" spans="1:27" x14ac:dyDescent="0.3">
@@ -9699,11 +9733,11 @@
       </c>
       <c r="T53" s="4">
         <f t="shared" si="17"/>
-        <v>-0.50382928908412938</v>
+        <v>-0.332334982552279</v>
       </c>
       <c r="U53" s="4">
         <f t="shared" si="18"/>
-        <v>-0.42276297064680413</v>
+        <v>-0.27886216128692509</v>
       </c>
       <c r="V53" s="4">
         <f t="shared" si="19"/>
@@ -9711,23 +9745,23 @@
       </c>
       <c r="W53" s="5">
         <f t="shared" si="25"/>
-        <v>0.65770242654952238</v>
+        <v>0.43383250872386064</v>
       </c>
       <c r="X53" s="2">
         <f t="shared" si="21"/>
-        <v>36772.026394926725</v>
+        <v>45276.332345085328</v>
       </c>
       <c r="Y53" s="1">
         <f t="shared" si="32"/>
-        <v>-972535407.0390383</v>
+        <v>-1580806468.6446433</v>
       </c>
       <c r="Z53" s="1">
         <f t="shared" si="33"/>
-        <v>676090962.59459388</v>
+        <v>1024973135.3113099</v>
       </c>
       <c r="AA53" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="54" spans="1:27" x14ac:dyDescent="0.3">
@@ -9806,11 +9840,11 @@
       </c>
       <c r="T54" s="4">
         <f t="shared" si="17"/>
-        <v>-0.47661281699888497</v>
+        <v>-0.3134446499564898</v>
       </c>
       <c r="U54" s="4">
         <f t="shared" si="18"/>
-        <v>-0.4766128169988848</v>
+        <v>-0.31344464995648968</v>
       </c>
       <c r="V54" s="4">
         <f t="shared" si="19"/>
@@ -9818,23 +9852,23 @@
       </c>
       <c r="W54" s="5">
         <f t="shared" si="25"/>
-        <v>0.67403230980066897</v>
+        <v>0.44327767502175514</v>
       </c>
       <c r="X54" s="2">
         <f t="shared" si="21"/>
-        <v>36323.854532502628</v>
+        <v>44791.370982607645</v>
       </c>
       <c r="Y54" s="1">
         <f t="shared" si="32"/>
-        <v>-956155648.49365032</v>
+        <v>-1558966790.5841265</v>
       </c>
       <c r="Z54" s="1">
         <f t="shared" si="33"/>
-        <v>659711204.0492059</v>
+        <v>1003133457.2507931</v>
       </c>
       <c r="AA54" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="55" spans="1:27" x14ac:dyDescent="0.3">
@@ -9913,11 +9947,11 @@
       </c>
       <c r="T55" s="4">
         <f t="shared" si="17"/>
-        <v>-0.44532606080535853</v>
+        <v>-0.29186799907667815</v>
       </c>
       <c r="U55" s="4">
         <f t="shared" si="18"/>
-        <v>-0.53071893284061344</v>
+        <v>-0.34783473646291463</v>
       </c>
       <c r="V55" s="4">
         <f t="shared" si="19"/>
@@ -9925,23 +9959,23 @@
       </c>
       <c r="W55" s="5">
         <f t="shared" si="25"/>
-        <v>0.69280436351678487</v>
+        <v>0.45406600046166096</v>
       </c>
       <c r="X55" s="2">
         <f t="shared" si="21"/>
-        <v>35828.36402358226</v>
+        <v>44256.064690000043</v>
       </c>
       <c r="Y55" s="1">
         <f t="shared" si="32"/>
-        <v>-938280278.74760628</v>
+        <v>-1535132964.2560678</v>
       </c>
       <c r="Z55" s="1">
         <f t="shared" si="33"/>
-        <v>641835834.30316186</v>
+        <v>979299630.92273426</v>
       </c>
       <c r="AA55" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333349</v>
       </c>
     </row>
     <row r="56" spans="1:27" x14ac:dyDescent="0.3">
@@ -10020,11 +10054,11 @@
       </c>
       <c r="T56" s="4">
         <f t="shared" si="17"/>
-        <v>-0.40965299566170249</v>
+        <v>-0.26744561144535206</v>
       </c>
       <c r="U56" s="4">
         <f t="shared" si="18"/>
-        <v>-0.58504510921019603</v>
+        <v>-0.38195191689760527</v>
       </c>
       <c r="V56" s="4">
         <f t="shared" si="19"/>
@@ -10032,23 +10066,23 @@
       </c>
       <c r="W56" s="5">
         <f t="shared" si="25"/>
-        <v>0.71420820260297846</v>
+        <v>0.46627719427732406</v>
       </c>
       <c r="X56" s="2">
         <f t="shared" si="21"/>
-        <v>35287.416899333191</v>
+        <v>43672.715650317623</v>
       </c>
       <c r="Y56" s="1">
         <f t="shared" si="32"/>
-        <v>-919045340.15811729</v>
+        <v>-1509486379.4700823</v>
       </c>
       <c r="Z56" s="1">
         <f t="shared" si="33"/>
-        <v>622600895.71367288</v>
+        <v>953653046.13674891</v>
       </c>
       <c r="AA56" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="57" spans="1:27" x14ac:dyDescent="0.3">
@@ -10127,11 +10161,11 @@
       </c>
       <c r="T57" s="4">
         <f t="shared" si="17"/>
-        <v>-0.36923076923076947</v>
+        <v>-0.24000000000000021</v>
       </c>
       <c r="U57" s="4">
         <f t="shared" si="18"/>
-        <v>-0.63952645202543124</v>
+        <v>-0.41569219381653039</v>
       </c>
       <c r="V57" s="4">
         <f t="shared" si="19"/>
@@ -10139,23 +10173,23 @@
       </c>
       <c r="W57" s="5">
         <f t="shared" si="25"/>
-        <v>0.73846153846153828</v>
+        <v>0.48</v>
       </c>
       <c r="X57" s="2">
         <f t="shared" si="21"/>
-        <v>34703.105848836582</v>
+        <v>43043.905233816527</v>
       </c>
       <c r="Y57" s="1">
         <f t="shared" si="32"/>
-        <v>-898597222.22222233</v>
+        <v>-1482222222.2222223</v>
       </c>
       <c r="Z57" s="1">
         <f t="shared" si="33"/>
-        <v>602152777.77777791</v>
+        <v>926388888.88888896</v>
       </c>
       <c r="AA57" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="58" spans="1:27" x14ac:dyDescent="0.3">
@@ -10234,11 +10268,11 @@
       </c>
       <c r="T58" s="4">
         <f t="shared" si="17"/>
-        <v>-0.32364624355021249</v>
+        <v>-0.20933628797318135</v>
       </c>
       <c r="U58" s="4">
         <f t="shared" si="18"/>
-        <v>-0.6940616090903533</v>
+        <v>-0.44892311827226966</v>
       </c>
       <c r="V58" s="4">
         <f t="shared" si="19"/>
@@ -10246,23 +10280,23 @@
       </c>
       <c r="W58" s="5">
         <f t="shared" si="25"/>
-        <v>0.76581225386987239</v>
+        <v>0.4953318560134094</v>
       </c>
       <c r="X58" s="2">
         <f t="shared" si="21"/>
-        <v>34077.767034237455</v>
+        <v>42372.506555037762</v>
       </c>
       <c r="Y58" s="1">
         <f t="shared" si="32"/>
-        <v>-877091547.46432495</v>
+        <v>-1453547989.2116923</v>
       </c>
       <c r="Z58" s="1">
         <f t="shared" si="33"/>
-        <v>580647103.01988053</v>
+        <v>897714655.87835908</v>
       </c>
       <c r="AA58" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="59" spans="1:27" x14ac:dyDescent="0.3">
@@ -10341,11 +10375,11 @@
       </c>
       <c r="T59" s="4">
         <f t="shared" si="17"/>
-        <v>-0.2724328285518825</v>
+        <v>-0.17524365585003041</v>
       </c>
       <c r="U59" s="4">
         <f t="shared" si="18"/>
-        <v>-0.74850304476445018</v>
+        <v>-0.48147798735063574</v>
       </c>
       <c r="V59" s="4">
         <f t="shared" si="19"/>
@@ -10353,23 +10387,23 @@
       </c>
       <c r="W59" s="5">
         <f t="shared" si="25"/>
-        <v>0.79654030286887045</v>
+        <v>0.51237817207498493</v>
       </c>
       <c r="X59" s="2">
         <f t="shared" si="21"/>
-        <v>33413.995349564822</v>
+        <v>41661.6988451586</v>
       </c>
       <c r="Y59" s="1">
         <f t="shared" si="32"/>
-        <v>-854691987.05481422</v>
+        <v>-1423681908.665678</v>
       </c>
       <c r="Z59" s="1">
         <f t="shared" si="33"/>
-        <v>558247542.6103698</v>
+        <v>867848575.33234477</v>
       </c>
       <c r="AA59" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="60" spans="1:27" x14ac:dyDescent="0.3">
@@ -10448,11 +10482,11 @@
       </c>
       <c r="T60" s="4">
         <f t="shared" si="17"/>
-        <v>-0.21506805770245746</v>
+        <v>-0.13749789067717394</v>
       </c>
       <c r="U60" s="4">
         <f t="shared" si="18"/>
-        <v>-0.80264491843072672</v>
+        <v>-0.51314911394076446</v>
       </c>
       <c r="V60" s="4">
         <f t="shared" si="19"/>
@@ -10460,23 +10494,23 @@
       </c>
       <c r="W60" s="5">
         <f t="shared" si="25"/>
-        <v>0.83095916537852543</v>
+        <v>0.53125105466141309</v>
       </c>
       <c r="X60" s="2">
         <f t="shared" si="21"/>
-        <v>32714.662484249679</v>
+        <v>40914.983713975351</v>
       </c>
       <c r="Y60" s="1">
         <f t="shared" si="32"/>
-        <v>-831569015.17363107</v>
+        <v>-1392851279.4907675</v>
       </c>
       <c r="Z60" s="1">
         <f t="shared" si="33"/>
-        <v>535124570.72918665</v>
+        <v>837017946.15743411</v>
       </c>
       <c r="AA60" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="61" spans="1:27" x14ac:dyDescent="0.3">
@@ -10555,11 +10589,11 @@
       </c>
       <c r="T61" s="4">
         <f t="shared" si="17"/>
-        <v>-0.15097258228534102</v>
+        <v>-9.5865474155977362E-2</v>
       </c>
       <c r="U61" s="4">
         <f t="shared" si="18"/>
-        <v>-0.85620806117559323</v>
+        <v>-0.54368012070982585</v>
       </c>
       <c r="V61" s="4">
         <f t="shared" si="19"/>
@@ -10567,23 +10601,23 @@
       </c>
       <c r="W61" s="5">
         <f t="shared" si="25"/>
-        <v>0.86941645062879536</v>
+        <v>0.55206726292201136</v>
       </c>
       <c r="X61" s="2">
         <f t="shared" si="21"/>
-        <v>31982.938175045107</v>
+        <v>40136.203309672681</v>
       </c>
       <c r="Y61" s="1">
         <f t="shared" si="32"/>
-        <v>-807898611.59882331</v>
+        <v>-1361290741.3910236</v>
       </c>
       <c r="Z61" s="1">
         <f t="shared" si="33"/>
-        <v>511454167.15437883</v>
+        <v>805457408.05769014</v>
       </c>
       <c r="AA61" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444448</v>
+        <v>-555833333.33333349</v>
       </c>
     </row>
     <row r="62" spans="1:27" x14ac:dyDescent="0.3">
@@ -10662,11 +10696,11 @@
       </c>
       <c r="T62" s="4">
         <f t="shared" si="17"/>
-        <v>-7.9511578622616139E-2</v>
+        <v>-5.0109768598056513E-2</v>
       </c>
       <c r="U62" s="4">
         <f t="shared" si="18"/>
-        <v>-0.9088215023316224</v>
+        <v>-0.57275727595505332</v>
       </c>
       <c r="V62" s="4">
         <f t="shared" si="19"/>
@@ -10674,23 +10708,23 @@
       </c>
       <c r="W62" s="5">
         <f t="shared" si="25"/>
-        <v>0.91229305282643014</v>
+        <v>0.57494511570097184</v>
       </c>
       <c r="X62" s="2">
         <f t="shared" si="21"/>
-        <v>31222.315031071324</v>
+        <v>39329.560276840792</v>
       </c>
       <c r="Y62" s="1">
         <f t="shared" si="32"/>
-        <v>-783860922.39417553</v>
+        <v>-1329240489.1181598</v>
       </c>
       <c r="Z62" s="1">
         <f t="shared" si="33"/>
-        <v>487416477.94973117</v>
+        <v>773407155.78482652</v>
       </c>
       <c r="AA62" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444436</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="63" spans="1:27" x14ac:dyDescent="0.3">
@@ -10769,11 +10803,11 @@
       </c>
       <c r="T63" s="4">
         <f t="shared" si="17"/>
-        <v>-1.7642137750684129E-16</v>
+        <v>-1.1026336094177581E-16</v>
       </c>
       <c r="U63" s="4">
         <f t="shared" si="18"/>
-        <v>-0.96</v>
+        <v>-0.60000000000000009</v>
       </c>
       <c r="V63" s="4">
         <f t="shared" si="19"/>
@@ -10781,23 +10815,23 @@
       </c>
       <c r="W63" s="5">
         <f t="shared" si="25"/>
-        <v>0.96</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="X63" s="2">
         <f t="shared" si="21"/>
-        <v>30436.637279582788</v>
+        <v>38499.63924794909</v>
       </c>
       <c r="Y63" s="1">
         <f t="shared" si="32"/>
-        <v>-759638888.88888884</v>
+        <v>-1296944444.4444442</v>
       </c>
       <c r="Z63" s="1">
         <f t="shared" si="33"/>
-        <v>463194444.44444436</v>
+        <v>741111111.11111093</v>
       </c>
       <c r="AA63" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444448</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="64" spans="1:27" x14ac:dyDescent="0.3">
@@ -10876,11 +10910,11 @@
       </c>
       <c r="T64" s="4">
         <f t="shared" si="17"/>
-        <v>8.8286308302482519E-2</v>
+        <v>5.4676114325910012E-2</v>
       </c>
       <c r="U64" s="4">
         <f t="shared" si="18"/>
-        <v>-1.0091171215150914</v>
+        <v>-0.62495084645691223</v>
       </c>
       <c r="V64" s="4">
         <f t="shared" si="19"/>
@@ -10888,23 +10922,23 @@
       </c>
       <c r="W64" s="5">
         <f t="shared" si="25"/>
-        <v>1.0129717849814894</v>
+        <v>0.6273380571629551</v>
       </c>
       <c r="X64" s="2">
         <f t="shared" si="21"/>
-        <v>29630.133679724022</v>
+        <v>37651.429360315007</v>
       </c>
       <c r="Y64" s="1">
         <f t="shared" si="32"/>
-        <v>-735416855.38360238</v>
+        <v>-1264648399.7707288</v>
       </c>
       <c r="Z64" s="1">
         <f t="shared" si="33"/>
-        <v>438972410.9391579</v>
+        <v>708815066.43739545</v>
       </c>
       <c r="AA64" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444448</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="65" spans="1:27" x14ac:dyDescent="0.3">
@@ -10983,11 +11017,11 @@
       </c>
       <c r="T65" s="4">
         <f t="shared" si="17"/>
-        <v>0.1860908530698959</v>
+        <v>0.11409511062010173</v>
       </c>
       <c r="U65" s="4">
         <f t="shared" si="18"/>
-        <v>-1.0553736718124533</v>
+        <v>-0.64706552656705585</v>
       </c>
       <c r="V65" s="4">
         <f t="shared" si="19"/>
@@ -10995,23 +11029,23 @@
       </c>
       <c r="W65" s="5">
         <f t="shared" si="25"/>
-        <v>1.0716545118419376</v>
+        <v>0.65704755531005099</v>
       </c>
       <c r="X65" s="2">
         <f t="shared" si="21"/>
-        <v>28807.454650993033</v>
+        <v>36790.346944940109</v>
       </c>
       <c r="Y65" s="1">
         <f t="shared" si="32"/>
-        <v>-711379166.17895448</v>
+        <v>-1232598147.4978654</v>
       </c>
       <c r="Z65" s="1">
         <f t="shared" si="33"/>
-        <v>414934721.73451006</v>
+        <v>676764814.16453207</v>
       </c>
       <c r="AA65" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="66" spans="1:27" x14ac:dyDescent="0.3">
@@ -11090,11 +11124,11 @@
       </c>
       <c r="T66" s="4">
         <f t="shared" si="17"/>
-        <v>0.29414438453498798</v>
+        <v>0.17837482844585298</v>
       </c>
       <c r="U66" s="4">
         <f t="shared" si="18"/>
-        <v>-1.0977617878456545</v>
+        <v>-0.66570392255130684</v>
       </c>
       <c r="V66" s="4">
         <f t="shared" si="19"/>
@@ -11102,23 +11136,23 @@
       </c>
       <c r="W66" s="5">
         <f t="shared" si="25"/>
-        <v>1.1364866307209929</v>
+        <v>0.68918741422292662</v>
       </c>
       <c r="X66" s="2">
         <f t="shared" si="21"/>
-        <v>27973.713309451869</v>
+        <v>35922.257057840565</v>
       </c>
       <c r="Y66" s="1">
         <f t="shared" si="32"/>
-        <v>-687708762.60414672</v>
+        <v>-1201037609.3981214</v>
       </c>
       <c r="Z66" s="1">
         <f t="shared" si="33"/>
-        <v>391264318.1597023</v>
+        <v>645204276.0647881</v>
       </c>
       <c r="AA66" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="67" spans="1:27" x14ac:dyDescent="0.3">
@@ -11197,11 +11231,11 @@
       </c>
       <c r="T67" s="4">
         <f t="shared" si="17"/>
-        <v>0.41311566495554747</v>
+        <v>0.24754472760245388</v>
       </c>
       <c r="U67" s="4">
         <f t="shared" si="18"/>
-        <v>-1.1350259610883469</v>
+        <v>-0.68012354939278685</v>
       </c>
       <c r="V67" s="4">
         <f t="shared" si="19"/>
@@ -11209,23 +11243,23 @@
       </c>
       <c r="W67" s="5">
         <f t="shared" si="25"/>
-        <v>1.2078693989733285</v>
+        <v>0.723772363801227</v>
       </c>
       <c r="X67" s="2">
         <f t="shared" si="21"/>
-        <v>27134.52952525689</v>
+        <v>35053.491891390135</v>
       </c>
       <c r="Y67" s="1">
         <f t="shared" si="32"/>
-        <v>-664585790.72296333</v>
+        <v>-1170206980.2232103</v>
       </c>
       <c r="Z67" s="1">
         <f t="shared" si="33"/>
-        <v>368141346.27851897</v>
+        <v>614373646.88987696</v>
       </c>
       <c r="AA67" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444436</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="68" spans="1:27" x14ac:dyDescent="0.3">
@@ -11304,11 +11338,11 @@
       </c>
       <c r="T68" s="4">
         <f t="shared" si="17"/>
-        <v>0.54353931575946934</v>
+        <v>0.3215086759204463</v>
       </c>
       <c r="U68" s="4">
         <f t="shared" si="18"/>
-        <v>-1.1656238242152115</v>
+        <v>-0.68947758051526165</v>
       </c>
       <c r="V68" s="4">
         <f t="shared" si="19"/>
@@ -11316,23 +11350,23 @@
       </c>
       <c r="W68" s="5">
         <f t="shared" si="25"/>
-        <v>1.2861235894556815</v>
+        <v>0.76075433796022329</v>
       </c>
       <c r="X68" s="2">
         <f t="shared" si="21"/>
-        <v>26296.075215476867</v>
+        <v>34190.86329251904</v>
       </c>
       <c r="Y68" s="1">
         <f t="shared" si="32"/>
-        <v>-642186230.31345272</v>
+        <v>-1140340899.6771963</v>
       </c>
       <c r="Z68" s="1">
         <f t="shared" si="33"/>
-        <v>345741785.86900836</v>
+        <v>584507566.34386289</v>
       </c>
       <c r="AA68" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444436</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="69" spans="1:27" x14ac:dyDescent="0.3">
@@ -11411,11 +11445,11 @@
       </c>
       <c r="T69" s="4">
         <f t="shared" si="17"/>
-        <v>0.68571428571428583</v>
+        <v>0.40000000000000019</v>
       </c>
       <c r="U69" s="4">
         <f t="shared" si="18"/>
-        <v>-1.1876919823329444</v>
+        <v>-0.69282032302755103</v>
       </c>
       <c r="V69" s="4">
         <f t="shared" si="19"/>
@@ -11423,23 +11457,23 @@
       </c>
       <c r="W69" s="5">
         <f t="shared" si="25"/>
-        <v>1.3714285714285714</v>
+        <v>0.80000000000000016</v>
       </c>
       <c r="X69" s="2">
         <f t="shared" si="21"/>
-        <v>25465.11775394377</v>
+        <v>33341.665625260328</v>
       </c>
       <c r="Y69" s="1">
         <f t="shared" si="32"/>
-        <v>-620680555.55555558</v>
+        <v>-1111666666.6666665</v>
       </c>
       <c r="Z69" s="1">
         <f t="shared" si="33"/>
-        <v>324236111.1111111</v>
+        <v>555833333.33333313</v>
       </c>
       <c r="AA69" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444448</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="70" spans="1:27" x14ac:dyDescent="0.3">
@@ -11518,11 +11552,11 @@
       </c>
       <c r="T70" s="4">
         <f t="shared" si="17"/>
-        <v>0.83956682871155941</v>
+        <v>0.48252969255536327</v>
       </c>
       <c r="U70" s="4">
         <f t="shared" si="18"/>
-        <v>-1.199025692951212</v>
+        <v>-0.68912381861682737</v>
       </c>
       <c r="V70" s="4">
         <f t="shared" si="19"/>
@@ -11530,23 +11564,23 @@
       </c>
       <c r="W70" s="5">
         <f t="shared" si="25"/>
-        <v>1.4637400972269357</v>
+        <v>0.84126484627768172</v>
       </c>
       <c r="X70" s="2">
         <f t="shared" si="21"/>
-        <v>24649.05650020772</v>
+        <v>32513.664084057749</v>
       </c>
       <c r="Y70" s="1">
         <f t="shared" si="32"/>
-        <v>-600232437.61966062</v>
+        <v>-1084402509.4188068</v>
       </c>
       <c r="Z70" s="1">
         <f t="shared" si="33"/>
-        <v>303787993.17521626</v>
+        <v>528569176.08547342</v>
       </c>
       <c r="AA70" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444436</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="71" spans="1:27" x14ac:dyDescent="0.3">
@@ -11625,11 +11659,11 @@
       </c>
       <c r="T71" s="4">
         <f t="shared" si="17"/>
-        <v>1.0044742770028396</v>
+        <v>0.56833045227777346</v>
       </c>
       <c r="U71" s="4">
         <f t="shared" si="18"/>
-        <v>-1.1970858282866059</v>
+        <v>-0.67730985828272894</v>
       </c>
       <c r="V71" s="4">
         <f t="shared" si="19"/>
@@ -11637,23 +11671,23 @@
       </c>
       <c r="W71" s="5">
         <f t="shared" si="25"/>
-        <v>1.5626845662017037</v>
+        <v>0.88416522613888682</v>
       </c>
       <c r="X71" s="2">
         <f t="shared" si="21"/>
-        <v>23855.944944006184</v>
+        <v>31715.062393111821</v>
       </c>
       <c r="Y71" s="1">
         <f t="shared" si="32"/>
-        <v>-580997499.03017151</v>
+        <v>-1058755924.6328212</v>
       </c>
       <c r="Z71" s="1">
         <f t="shared" si="33"/>
-        <v>284553054.5857271</v>
+        <v>502922591.29948783</v>
       </c>
       <c r="AA71" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="72" spans="1:27" x14ac:dyDescent="0.3">
@@ -11732,11 +11766,11 @@
       </c>
       <c r="T72" s="4">
         <f t="shared" si="17"/>
-        <v>1.179051841389128</v>
+        <v>0.65630179281363243</v>
       </c>
       <c r="U72" s="4">
         <f t="shared" si="18"/>
-        <v>-1.1790518413891287</v>
+        <v>-0.65630179281363277</v>
       </c>
       <c r="V72" s="4">
         <f t="shared" si="19"/>
@@ -11744,23 +11778,23 @@
       </c>
       <c r="W72" s="5">
         <f t="shared" si="25"/>
-        <v>1.6674311048334767</v>
+        <v>0.92815089640681636</v>
       </c>
       <c r="X72" s="2">
         <f t="shared" si="21"/>
-        <v>23094.487863543683</v>
+        <v>30954.442814285296</v>
       </c>
       <c r="Y72" s="1">
         <f t="shared" si="32"/>
-        <v>-563122129.28412771</v>
+        <v>-1034922098.3047626</v>
       </c>
       <c r="Z72" s="1">
         <f t="shared" si="33"/>
-        <v>266677684.83968323</v>
+        <v>479088764.97142929</v>
       </c>
       <c r="AA72" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444448</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="73" spans="1:27" x14ac:dyDescent="0.3">
@@ -11839,11 +11873,11 @@
       </c>
       <c r="T73" s="4">
         <f t="shared" si="17"/>
-        <v>1.3609159056305076</v>
+        <v>0.74496470040323171</v>
       </c>
       <c r="U73" s="4">
         <f t="shared" si="18"/>
-        <v>-1.1419440344778538</v>
+        <v>-0.625099605348445</v>
       </c>
       <c r="V73" s="4">
         <f t="shared" si="19"/>
@@ -11851,23 +11885,23 @@
       </c>
       <c r="W73" s="5">
         <f t="shared" si="25"/>
-        <v>1.7765495433783045</v>
+        <v>0.972482350201616</v>
       </c>
       <c r="X73" s="2">
         <f t="shared" si="21"/>
-        <v>22373.999476816622</v>
+        <v>30240.670856014818</v>
       </c>
       <c r="Y73" s="1">
         <f t="shared" si="32"/>
-        <v>-546742370.73873961</v>
+        <v>-1013082420.2442453</v>
       </c>
       <c r="Z73" s="1">
         <f t="shared" si="33"/>
-        <v>250297926.29429522</v>
+        <v>457249086.91091198</v>
       </c>
       <c r="AA73" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="74" spans="1:27" x14ac:dyDescent="0.3">
@@ -11946,11 +11980,11 @@
       </c>
       <c r="T74" s="4">
         <f t="shared" ref="T74:T81" si="45">W74*COS(RADIANS(S74))*(COS($Y$5)*COS($Y$6))+W74*SIN(RADIANS(S74))*(COS($Y$5)*SIN($Y$6)*SIN($Y$7)-SIN($Y$5)*COS($Y$7))</f>
-        <v>1.5464550537021047</v>
+        <v>0.83243778201311258</v>
       </c>
       <c r="U74" s="4">
         <f t="shared" ref="U74:U81" si="46">W74*COS(RADIANS(S74))*(SIN(Y$5)*COS(Y$6))+W74*SIN(RADIANS(S74))*(SIN(Y$5)*SIN(Y$6)*SIN(Y$7)+COS(Y$5)*COS(Y$7))</f>
-        <v>-1.0828394861047161</v>
+        <v>-0.58287921005615317</v>
       </c>
       <c r="V74" s="4">
         <f t="shared" ref="V74:V81" si="47">W74*COS(RADIANS(S74))*(-SIN(Y$6))+W74*SIN(RADIANS(S74))*(COS(Y$6)*SIN(Y$7))</f>
@@ -11958,23 +11992,23 @@
       </c>
       <c r="W74" s="5">
         <f t="shared" si="25"/>
-        <v>1.8878730322212627</v>
+        <v>1.0162188910065564</v>
       </c>
       <c r="X74" s="2">
         <f t="shared" ref="X74:X81" si="48">SQRT(0.0000000000667*2E+30/(W74*150000000000))</f>
-        <v>21704.305508468231</v>
+        <v>29582.757486587849</v>
       </c>
       <c r="Y74" s="1">
         <f t="shared" si="32"/>
-        <v>-531982883.24690664</v>
+        <v>-993403103.58846807</v>
       </c>
       <c r="Z74" s="1">
         <f t="shared" si="33"/>
-        <v>235538438.80246219</v>
+        <v>437569770.2551347</v>
       </c>
       <c r="AA74" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="75" spans="1:27" x14ac:dyDescent="0.3">
@@ -12053,11 +12087,11 @@
       </c>
       <c r="T75" s="4">
         <f t="shared" si="45"/>
-        <v>1.7306635447028222</v>
+        <v>0.91644952894850817</v>
       </c>
       <c r="U75" s="4">
         <f t="shared" si="46"/>
-        <v>-0.99919906341084752</v>
+        <v>-0.52911238223712753</v>
       </c>
       <c r="V75" s="4">
         <f t="shared" si="47"/>
@@ -12065,23 +12099,23 @@
       </c>
       <c r="W75" s="5">
         <f t="shared" si="25"/>
-        <v>1.9983981268216933</v>
+        <v>1.0582247644742542</v>
       </c>
       <c r="X75" s="2">
         <f t="shared" si="48"/>
-        <v>21095.570671400161</v>
+        <v>28989.673557546113</v>
       </c>
       <c r="Y75" s="1">
         <f t="shared" si="32"/>
-        <v>-518955995.42046374</v>
+        <v>-976033919.81987762</v>
       </c>
       <c r="Z75" s="1">
         <f t="shared" si="33"/>
-        <v>222511550.97601932</v>
+        <v>420200586.48654419</v>
       </c>
       <c r="AA75" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333349</v>
       </c>
     </row>
     <row r="76" spans="1:27" x14ac:dyDescent="0.3">
@@ -12160,11 +12194,11 @@
       </c>
       <c r="T76" s="4">
         <f t="shared" si="45"/>
-        <v>1.9071158345178281</v>
+        <v>0.99440165299999717</v>
       </c>
       <c r="U76" s="4">
         <f t="shared" si="46"/>
-        <v>-0.88930271862432375</v>
+        <v>-0.46369710607588793</v>
       </c>
       <c r="V76" s="4">
         <f t="shared" si="47"/>
@@ -12172,23 +12206,23 @@
       </c>
       <c r="W76" s="5">
         <f t="shared" si="25"/>
-        <v>2.1042695007106968</v>
+        <v>1.0972008264999986</v>
       </c>
       <c r="X76" s="2">
         <f t="shared" si="48"/>
-        <v>20558.035183216096</v>
+        <v>28470.115053558147</v>
       </c>
       <c r="Y76" s="1">
         <f t="shared" si="32"/>
-        <v>-507760849.74161983</v>
+        <v>-961107058.91475248</v>
       </c>
       <c r="Z76" s="1">
         <f t="shared" si="33"/>
-        <v>211316405.29717544</v>
+        <v>405273725.58141911</v>
       </c>
       <c r="AA76" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="77" spans="1:27" x14ac:dyDescent="0.3">
@@ -12267,11 +12301,11 @@
       </c>
       <c r="T77" s="4">
         <f t="shared" si="45"/>
-        <v>2.0681731373723151</v>
+        <v>1.0634945743553152</v>
       </c>
       <c r="U77" s="4">
         <f t="shared" si="46"/>
-        <v>-0.7527534613124679</v>
+        <v>-0.38708036936893914</v>
       </c>
       <c r="V77" s="4">
         <f t="shared" si="47"/>
@@ -12279,23 +12313,23 @@
       </c>
       <c r="W77" s="5">
         <f t="shared" ref="W77:W81" si="49">W$3/(1-T$6*COS(RADIANS(S77)))</f>
-        <v>2.2009038824233889</v>
+        <v>1.1317472871776577</v>
       </c>
       <c r="X77" s="2">
         <f t="shared" si="48"/>
-        <v>20101.651851743965</v>
+        <v>28032.223956166334</v>
       </c>
       <c r="Y77" s="1">
         <f t="shared" si="32"/>
-        <v>-498482648.02880526</v>
+        <v>-948736123.29766619</v>
       </c>
       <c r="Z77" s="1">
         <f t="shared" si="33"/>
-        <v>202038203.58436081</v>
+        <v>392902789.96433282</v>
       </c>
       <c r="AA77" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="78" spans="1:27" x14ac:dyDescent="0.3">
@@ -12374,11 +12408,11 @@
       </c>
       <c r="T78" s="4">
         <f t="shared" si="45"/>
-        <v>2.2054962876570996</v>
+        <v>1.1209166818152287</v>
       </c>
       <c r="U78" s="4">
         <f t="shared" si="46"/>
-        <v>-0.5909609491875587</v>
+        <v>-0.30034871967496418</v>
       </c>
       <c r="V78" s="4">
         <f t="shared" si="47"/>
@@ -12386,23 +12420,23 @@
       </c>
       <c r="W78" s="5">
         <f t="shared" si="49"/>
-        <v>2.2832977725942598</v>
+        <v>1.1604583409076143</v>
       </c>
       <c r="X78" s="2">
         <f t="shared" si="48"/>
-        <v>19735.630648902043</v>
+        <v>27683.277621159901</v>
       </c>
       <c r="Y78" s="1">
         <f t="shared" si="32"/>
-        <v>-491192002.99938524</v>
+        <v>-939015263.25843966</v>
       </c>
       <c r="Z78" s="1">
         <f t="shared" si="33"/>
-        <v>194747558.55494082</v>
+        <v>383181929.92510629</v>
       </c>
       <c r="AA78" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="79" spans="1:27" x14ac:dyDescent="0.3">
@@ -12481,11 +12515,11 @@
       </c>
       <c r="T79" s="4">
         <f t="shared" si="45"/>
-        <v>2.3108774751869507</v>
+        <v>1.1640842482013765</v>
       </c>
       <c r="U79" s="4">
         <f t="shared" si="46"/>
-        <v>-0.40747004798691583</v>
+        <v>-0.20525946077563212</v>
       </c>
       <c r="V79" s="4">
         <f t="shared" si="47"/>
@@ -12493,23 +12527,23 @@
       </c>
       <c r="W79" s="5">
         <f t="shared" si="49"/>
-        <v>2.3465264851121703</v>
+        <v>1.1820421241006884</v>
       </c>
       <c r="X79" s="2">
         <f t="shared" si="48"/>
-        <v>19467.920095367233</v>
+        <v>27429.368460766789</v>
       </c>
       <c r="Y79" s="1">
         <f t="shared" si="32"/>
-        <v>-485944400.86424613</v>
+        <v>-932018460.41158724</v>
       </c>
       <c r="Z79" s="1">
         <f t="shared" si="33"/>
-        <v>189499956.41980168</v>
+        <v>376185127.07825392</v>
       </c>
       <c r="AA79" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
     <row r="80" spans="1:27" x14ac:dyDescent="0.3">
@@ -12588,11 +12622,11 @@
       </c>
       <c r="T80" s="4">
         <f t="shared" si="45"/>
-        <v>2.3772977717989163</v>
+        <v>1.1909018964509861</v>
       </c>
       <c r="U80" s="4">
         <f t="shared" si="46"/>
-        <v>-0.20798660485784459</v>
+        <v>-0.10419041531098529</v>
       </c>
       <c r="V80" s="4">
         <f t="shared" si="47"/>
@@ -12600,23 +12634,23 @@
       </c>
       <c r="W80" s="5">
         <f t="shared" si="49"/>
-        <v>2.3863786630793498</v>
+        <v>1.1954509482254931</v>
       </c>
       <c r="X80" s="2">
         <f t="shared" si="48"/>
-        <v>19304.679981796133</v>
+        <v>27275.103347860128</v>
       </c>
       <c r="Y80" s="1">
         <f t="shared" si="32"/>
-        <v>-482779779.04422462</v>
+        <v>-927798964.65155876</v>
       </c>
       <c r="Z80" s="1">
         <f t="shared" si="33"/>
-        <v>186335334.59978017</v>
+        <v>371965631.31822538</v>
       </c>
       <c r="AA80" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333337</v>
       </c>
     </row>
     <row r="81" spans="1:27" x14ac:dyDescent="0.3">
@@ -12695,11 +12729,11 @@
       </c>
       <c r="T81" s="4">
         <f t="shared" si="45"/>
-        <v>2.4</v>
+        <v>1.2000000000000002</v>
       </c>
       <c r="U81" s="4">
         <f t="shared" si="46"/>
-        <v>-5.8807125835613761E-16</v>
+        <v>-2.9403562917806885E-16</v>
       </c>
       <c r="V81" s="4">
         <f t="shared" si="47"/>
@@ -12707,23 +12741,23 @@
       </c>
       <c r="W81" s="5">
         <f t="shared" si="49"/>
-        <v>2.4</v>
+        <v>1.2000000000000002</v>
       </c>
       <c r="X81" s="2">
         <f t="shared" si="48"/>
-        <v>19249.819623974548</v>
+        <v>27223.355985460556</v>
       </c>
       <c r="Y81" s="1">
         <f t="shared" si="32"/>
-        <v>-481722222.22222221</v>
+        <v>-926388888.88888884</v>
       </c>
       <c r="Z81" s="1">
         <f t="shared" si="33"/>
-        <v>185277777.77777782</v>
+        <v>370555555.55555552</v>
       </c>
       <c r="AA81" s="1">
         <f t="shared" si="34"/>
-        <v>-296444444.44444442</v>
+        <v>-555833333.33333325</v>
       </c>
     </row>
   </sheetData>

</xml_diff>